<commit_message>
style footer mẫu chi hoa hồng
</commit_message>
<xml_diff>
--- a/public/templates/mau-chi-hoa-hong-text.xlsx
+++ b/public/templates/mau-chi-hoa-hong-text.xlsx
@@ -206,7 +206,7 @@
     <t>HOA HỒNG DL HƯỞNG</t>
   </si>
   <si>
-    <t>M-INVOICE CÒN PHẢI THU</t>
+    <t xml:space="preserve">CÔNG NỢ TỔNG CỘNG ( Âm - M-invoice chi ; Dương - M-invoice thu) </t>
   </si>
   <si>
     <t>Giám đốc kinh doanh</t>
@@ -492,7 +492,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -515,6 +515,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.4"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -969,7 +975,7 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -993,16 +999,16 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1011,16 +1017,16 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1029,67 +1035,67 @@
     <xf numFmtId="0" fontId="32" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="31" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
@@ -1103,7 +1109,7 @@
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1214,8 +1220,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="57" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="57" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="57" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="57" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1240,7 +1249,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="10" fillId="0" borderId="10" xfId="53" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1258,7 +1267,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="179" fontId="1" fillId="6" borderId="1" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="1" fillId="7" borderId="1" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="179" fontId="12" fillId="3" borderId="11" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1276,6 +1285,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="179" fontId="3" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="179" fontId="3" fillId="5" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="51" applyFont="1" applyFill="1"/>
     <xf numFmtId="37" fontId="3" fillId="2" borderId="9" xfId="51" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1568,6 +1579,11 @@
       <tableStyleElement type="pageFieldValues" dxfId="8"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="005C1859"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1961,14 +1977,14 @@
       <c r="F3" s="10"/>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
-      <c r="M3" s="49"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="51"/>
-      <c r="P3" s="50"/>
+      <c r="M3" s="50"/>
+      <c r="N3" s="51"/>
+      <c r="O3" s="52"/>
+      <c r="P3" s="51"/>
     </row>
     <row r="4" s="2" customFormat="1" ht="15.6" spans="4:13">
       <c r="D4" s="11"/>
-      <c r="M4" s="49"/>
+      <c r="M4" s="50"/>
     </row>
     <row r="5" s="3" customFormat="1" ht="28.9" customHeight="1" spans="2:19">
       <c r="B5" s="12"/>
@@ -1986,7 +2002,7 @@
       <c r="L5" s="12"/>
       <c r="M5" s="12"/>
       <c r="N5" s="12"/>
-      <c r="O5" s="52"/>
+      <c r="O5" s="53"/>
       <c r="P5" s="12"/>
       <c r="Q5" s="12"/>
       <c r="R5" s="12"/>
@@ -2060,31 +2076,31 @@
       <c r="I8" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="53" t="s">
+      <c r="J8" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="K8" s="54" t="s">
+      <c r="K8" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="L8" s="54" t="s">
+      <c r="L8" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="M8" s="53" t="s">
+      <c r="M8" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="N8" s="53" t="s">
+      <c r="N8" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="O8" s="53" t="s">
+      <c r="O8" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="P8" s="53" t="s">
+      <c r="P8" s="54" t="s">
         <v>21</v>
       </c>
-      <c r="Q8" s="53" t="s">
+      <c r="Q8" s="54" t="s">
         <v>22</v>
       </c>
-      <c r="R8" s="68" t="s">
+      <c r="R8" s="71" t="s">
         <v>23</v>
       </c>
       <c r="S8" s="14" t="s">
@@ -2192,20 +2208,20 @@
       <c r="K10" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="L10" s="55" t="e">
+      <c r="L10" s="56" t="e">
         <f t="shared" ref="L10:L14" si="5">E10+I10+J10</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M10" s="56" t="s">
+      <c r="M10" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="N10" s="55" t="s">
+      <c r="N10" s="56" t="s">
         <v>38</v>
       </c>
       <c r="O10" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="P10" s="55" t="e">
+      <c r="P10" s="56" t="e">
         <f t="shared" ref="P10:P14" si="6">N10+M10-O10</f>
         <v>#VALUE!</v>
       </c>
@@ -2293,21 +2309,21 @@
       <c r="F12" s="22"/>
       <c r="G12" s="24"/>
       <c r="H12" s="25"/>
-      <c r="I12" s="55"/>
+      <c r="I12" s="56"/>
       <c r="J12" s="25"/>
       <c r="K12" s="22"/>
-      <c r="L12" s="55">
+      <c r="L12" s="56">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="M12" s="25"/>
-      <c r="N12" s="55"/>
+      <c r="N12" s="56"/>
       <c r="O12" s="25"/>
-      <c r="P12" s="55">
+      <c r="P12" s="56">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Q12" s="55"/>
+      <c r="Q12" s="56"/>
       <c r="R12" s="25"/>
       <c r="S12" s="25"/>
     </row>
@@ -2377,7 +2393,7 @@
         <v>0</v>
       </c>
       <c r="S13" s="23"/>
-      <c r="T13" s="69"/>
+      <c r="T13" s="72"/>
     </row>
     <row r="14" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
       <c r="A14" s="18"/>
@@ -2391,18 +2407,18 @@
       <c r="I14" s="25"/>
       <c r="J14" s="25"/>
       <c r="K14" s="22"/>
-      <c r="L14" s="55">
+      <c r="L14" s="56">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="M14" s="56"/>
-      <c r="N14" s="55"/>
+      <c r="M14" s="57"/>
+      <c r="N14" s="56"/>
       <c r="O14" s="25"/>
-      <c r="P14" s="55">
+      <c r="P14" s="56">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="Q14" s="55"/>
+      <c r="Q14" s="56"/>
       <c r="R14" s="25"/>
       <c r="S14" s="25"/>
     </row>
@@ -2472,7 +2488,7 @@
         <v>0</v>
       </c>
       <c r="S15" s="23"/>
-      <c r="T15" s="69"/>
+      <c r="T15" s="72"/>
     </row>
     <row r="16" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
       <c r="A16" s="18"/>
@@ -2486,14 +2502,14 @@
       <c r="I16" s="22"/>
       <c r="J16" s="22"/>
       <c r="K16" s="22"/>
-      <c r="L16" s="55">
+      <c r="L16" s="56">
         <f t="shared" ref="L16:L20" si="11">E16+I16+J16</f>
         <v>0</v>
       </c>
-      <c r="M16" s="56"/>
-      <c r="N16" s="55"/>
+      <c r="M16" s="57"/>
+      <c r="N16" s="56"/>
       <c r="O16" s="25"/>
-      <c r="P16" s="55">
+      <c r="P16" s="56">
         <f t="shared" ref="P16:P20" si="12">N16+M16-O16</f>
         <v>0</v>
       </c>
@@ -2567,7 +2583,7 @@
         <v>0</v>
       </c>
       <c r="S17" s="23"/>
-      <c r="T17" s="69"/>
+      <c r="T17" s="72"/>
     </row>
     <row r="18" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
       <c r="A18" s="18"/>
@@ -2581,14 +2597,14 @@
       <c r="I18" s="22"/>
       <c r="J18" s="22"/>
       <c r="K18" s="22"/>
-      <c r="L18" s="55">
+      <c r="L18" s="56">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="M18" s="56"/>
-      <c r="N18" s="55"/>
+      <c r="M18" s="57"/>
+      <c r="N18" s="56"/>
       <c r="O18" s="25"/>
-      <c r="P18" s="55">
+      <c r="P18" s="56">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
@@ -2610,7 +2626,7 @@
       <c r="G19" s="29"/>
       <c r="H19" s="29"/>
       <c r="I19" s="29"/>
-      <c r="J19" s="57"/>
+      <c r="J19" s="58"/>
       <c r="K19" s="23">
         <f>SUM(K20:K20)</f>
         <v>0</v>
@@ -2665,24 +2681,24 @@
       <c r="G20" s="32"/>
       <c r="H20" s="33"/>
       <c r="I20" s="32"/>
-      <c r="J20" s="58"/>
+      <c r="J20" s="59"/>
       <c r="K20" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="L20" s="55" t="e">
+      <c r="L20" s="56" t="e">
         <f t="shared" si="11"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M20" s="56" t="s">
+      <c r="M20" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="N20" s="55" t="s">
+      <c r="N20" s="56" t="s">
         <v>38</v>
       </c>
       <c r="O20" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="P20" s="55" t="e">
+      <c r="P20" s="56" t="e">
         <f>N20+M20-O20</f>
         <v>#VALUE!</v>
       </c>
@@ -2772,15 +2788,15 @@
       <c r="H22" s="36"/>
       <c r="I22" s="36"/>
       <c r="J22" s="36"/>
-      <c r="K22" s="59"/>
-      <c r="L22" s="55">
+      <c r="K22" s="60"/>
+      <c r="L22" s="56">
         <f>E22+I22+J22</f>
         <v>0</v>
       </c>
       <c r="M22" s="25"/>
-      <c r="N22" s="60"/>
+      <c r="N22" s="61"/>
       <c r="O22" s="25"/>
-      <c r="P22" s="55">
+      <c r="P22" s="56">
         <f>N22+M22-O22</f>
         <v>0</v>
       </c>
@@ -2800,40 +2816,40 @@
       <c r="G23" s="41"/>
       <c r="H23" s="41"/>
       <c r="I23" s="41"/>
-      <c r="J23" s="61"/>
-      <c r="K23" s="62">
+      <c r="J23" s="62"/>
+      <c r="K23" s="63">
         <f ca="1" t="shared" ref="K23:R23" si="17">K9+K11+K13+K15+K17+K19+K21</f>
         <v>0</v>
       </c>
-      <c r="L23" s="62" t="e">
+      <c r="L23" s="63" t="e">
         <f t="shared" si="17"/>
         <v>#VALUE!</v>
       </c>
-      <c r="M23" s="62">
+      <c r="M23" s="63">
         <f ca="1" t="shared" si="17"/>
         <v>0</v>
       </c>
-      <c r="N23" s="62">
+      <c r="N23" s="63">
         <f ca="1" t="shared" si="17"/>
         <v>0</v>
       </c>
-      <c r="O23" s="62">
+      <c r="O23" s="63">
         <f ca="1" t="shared" si="17"/>
         <v>0</v>
       </c>
-      <c r="P23" s="62" t="e">
+      <c r="P23" s="63" t="e">
         <f t="shared" si="17"/>
         <v>#VALUE!</v>
       </c>
-      <c r="Q23" s="62">
+      <c r="Q23" s="63">
         <f ca="1" t="shared" si="17"/>
         <v>0</v>
       </c>
-      <c r="R23" s="62">
+      <c r="R23" s="63">
         <f ca="1" t="shared" si="17"/>
         <v>0</v>
       </c>
-      <c r="S23" s="62"/>
+      <c r="S23" s="63"/>
     </row>
     <row r="24" s="6" customFormat="1" ht="33" customHeight="1" spans="3:19">
       <c r="C24" s="42" t="s">
@@ -2844,15 +2860,15 @@
       <c r="F24" s="42"/>
       <c r="G24" s="42"/>
       <c r="H24" s="43"/>
-      <c r="M24" s="63">
+      <c r="M24" s="64">
         <f ca="1">N23</f>
         <v>0</v>
       </c>
-      <c r="N24" s="63"/>
-      <c r="O24" s="64"/>
-      <c r="P24" s="64"/>
-      <c r="Q24" s="67"/>
-      <c r="S24" s="67"/>
+      <c r="N24" s="64"/>
+      <c r="O24" s="65"/>
+      <c r="P24" s="65"/>
+      <c r="Q24" s="68"/>
+      <c r="S24" s="68"/>
     </row>
     <row r="25" s="6" customFormat="1" ht="33" customHeight="1" spans="3:18">
       <c r="C25" s="43" t="s">
@@ -2863,15 +2879,15 @@
       <c r="F25" s="43"/>
       <c r="G25" s="43"/>
       <c r="H25" s="43"/>
-      <c r="M25" s="65">
+      <c r="M25" s="66">
         <f ca="1">M24*10%</f>
         <v>0</v>
       </c>
-      <c r="N25" s="65"/>
-      <c r="O25" s="64"/>
-      <c r="P25" s="66"/>
-      <c r="Q25" s="66"/>
-      <c r="R25" s="67"/>
+      <c r="N25" s="66"/>
+      <c r="O25" s="65"/>
+      <c r="P25" s="67"/>
+      <c r="Q25" s="67"/>
+      <c r="R25" s="68"/>
     </row>
     <row r="26" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
       <c r="C26" s="43" t="s">
@@ -2882,94 +2898,97 @@
       <c r="F26" s="43"/>
       <c r="G26" s="43"/>
       <c r="H26" s="43"/>
-      <c r="I26" s="67"/>
-      <c r="M26" s="65">
+      <c r="I26" s="68"/>
+      <c r="M26" s="66">
         <f ca="1">M24-M25</f>
-        <v>210000</v>
-      </c>
-      <c r="N26" s="65"/>
-      <c r="O26" s="64"/>
-      <c r="P26" s="66"/>
-      <c r="Q26" s="66"/>
+        <v>0</v>
+      </c>
+      <c r="N26" s="66"/>
+      <c r="O26" s="65"/>
+      <c r="P26" s="67"/>
+      <c r="Q26" s="67"/>
     </row>
     <row r="27" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
       <c r="C27" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="43"/>
-      <c r="I27" s="67"/>
-      <c r="M27" s="65">
+      <c r="D27" s="44"/>
+      <c r="E27" s="44"/>
+      <c r="F27" s="44"/>
+      <c r="G27" s="44"/>
+      <c r="H27" s="45"/>
+      <c r="I27" s="69"/>
+      <c r="J27" s="70"/>
+      <c r="K27" s="70"/>
+      <c r="L27" s="70"/>
+      <c r="M27" s="66">
         <f ca="1">R23-M26</f>
-        <v>-210000</v>
-      </c>
-      <c r="N27" s="65"/>
-      <c r="O27" s="64"/>
-      <c r="P27" s="66"/>
-      <c r="Q27" s="66"/>
+        <v>0</v>
+      </c>
+      <c r="N27" s="66"/>
+      <c r="O27" s="65"/>
+      <c r="P27" s="67"/>
+      <c r="Q27" s="67"/>
     </row>
     <row r="28" s="7" customFormat="1" ht="33" customHeight="1" spans="1:18">
-      <c r="A28" s="45" t="s">
+      <c r="A28" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="B28" s="45"/>
-      <c r="C28" s="45"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="46"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="47"/>
-      <c r="H28" s="47"/>
-      <c r="I28" s="47"/>
-      <c r="J28" s="47"/>
-      <c r="M28" s="47"/>
-      <c r="N28" s="47"/>
-      <c r="O28" s="47"/>
-      <c r="P28" s="47"/>
-      <c r="Q28" s="47" t="s">
+      <c r="B28" s="46"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="48"/>
+      <c r="H28" s="48"/>
+      <c r="I28" s="48"/>
+      <c r="J28" s="48"/>
+      <c r="M28" s="48"/>
+      <c r="N28" s="48"/>
+      <c r="O28" s="48"/>
+      <c r="P28" s="48"/>
+      <c r="Q28" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="R28" s="47"/>
+      <c r="R28" s="48"/>
     </row>
     <row r="29" s="1" customFormat="1" ht="33" customHeight="1"/>
     <row r="30" s="1" customFormat="1" ht="33" customHeight="1"/>
     <row r="32" s="1" customFormat="1" spans="18:18">
-      <c r="R32" s="70"/>
+      <c r="R32" s="73"/>
     </row>
     <row r="35" s="1" customFormat="1" spans="1:18">
-      <c r="A35" s="47" t="s">
+      <c r="A35" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="B35" s="47"/>
-      <c r="C35" s="47"/>
-      <c r="D35" s="47"/>
-      <c r="G35" s="47"/>
-      <c r="H35" s="47"/>
-      <c r="I35" s="47"/>
-      <c r="J35" s="47"/>
+      <c r="B35" s="48"/>
+      <c r="C35" s="48"/>
+      <c r="D35" s="48"/>
+      <c r="G35" s="48"/>
+      <c r="H35" s="48"/>
+      <c r="I35" s="48"/>
+      <c r="J35" s="48"/>
       <c r="K35" s="7"/>
-      <c r="M35" s="47"/>
-      <c r="N35" s="47"/>
-      <c r="O35" s="47"/>
-      <c r="P35" s="47"/>
-      <c r="Q35" s="47" t="s">
+      <c r="M35" s="48"/>
+      <c r="N35" s="48"/>
+      <c r="O35" s="48"/>
+      <c r="P35" s="48"/>
+      <c r="Q35" s="48" t="s">
         <v>63</v>
       </c>
-      <c r="R35" s="47"/>
+      <c r="R35" s="48"/>
     </row>
     <row r="36" s="4" customFormat="1" spans="3:14">
-      <c r="C36" s="48"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="48"/>
-      <c r="F36" s="48"/>
-      <c r="G36" s="48"/>
-      <c r="H36" s="48"/>
-      <c r="N36" s="64"/>
+      <c r="C36" s="49"/>
+      <c r="D36" s="49"/>
+      <c r="E36" s="49"/>
+      <c r="F36" s="49"/>
+      <c r="G36" s="49"/>
+      <c r="H36" s="49"/>
+      <c r="N36" s="65"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="23">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="E19:J19"/>
     <mergeCell ref="E20:J20"/>
@@ -2982,6 +3001,7 @@
     <mergeCell ref="C26:G26"/>
     <mergeCell ref="M26:N26"/>
     <mergeCell ref="P26:Q26"/>
+    <mergeCell ref="C27:G27"/>
     <mergeCell ref="M27:N27"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="G28:J28"/>

</xml_diff>

<commit_message>
cập nhật thêm danh mục xăng dầu
</commit_message>
<xml_diff>
--- a/public/templates/mau-chi-hoa-hong-text.xlsx
+++ b/public/templates/mau-chi-hoa-hong-text.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="66">
   <si>
     <t>CÔNG TY TNHH HÓA ĐƠN ĐIỆN TỬ M-INVOICE - CHI NHÁNH TP. HỒ CHÍ MINH</t>
   </si>
@@ -179,10 +179,16 @@
     <t>E. QUẢN LÝ HÓA ĐƠN SMI</t>
   </si>
   <si>
+    <t>XANG</t>
+  </si>
+  <si>
+    <t>F. XĂNG DẦU</t>
+  </si>
+  <si>
     <t>CKS</t>
   </si>
   <si>
-    <t>F. GIÁ TRỊ CHỮ KÝ SỐ</t>
+    <t>G. GIÁ TRỊ CHỮ KÝ SỐ</t>
   </si>
   <si>
     <t>TÊN SP</t>
@@ -191,7 +197,7 @@
     <t>KHAC</t>
   </si>
   <si>
-    <t>F. KHAC</t>
+    <t>H. KHAC</t>
   </si>
   <si>
     <t>CỘNG</t>
@@ -1921,7 +1927,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:T36"/>
+  <dimension ref="A1:T38"/>
   <sheetFormatPr defaultColWidth="7.71296296296296" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="5.28703703703704" style="1" customWidth="1"/>
@@ -2621,22 +2627,40 @@
       <c r="D19" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="28"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="29"/>
-      <c r="J19" s="58"/>
+      <c r="E19" s="23">
+        <f t="shared" ref="E19:R19" si="14">SUM(E20:E20)</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="23">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="G19" s="23">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="H19" s="23">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="I19" s="23">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="J19" s="23">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
       <c r="K19" s="23">
-        <f>SUM(K20:K20)</f>
-        <v>0</v>
-      </c>
-      <c r="L19" s="23" t="e">
-        <f>SUM(L20:L20)</f>
-        <v>#VALUE!</v>
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="L19" s="23">
+        <f t="shared" si="14"/>
+        <v>0</v>
       </c>
       <c r="M19" s="23">
-        <f t="shared" ref="M19:S19" si="14">SUM(M20:M20)</f>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="N19" s="23">
@@ -2647,9 +2671,9 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="P19" s="23" t="e">
+      <c r="P19" s="23">
         <f t="shared" si="14"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="23">
         <f t="shared" si="14"/>
@@ -2661,357 +2685,433 @@
       </c>
       <c r="S19" s="23"/>
     </row>
-    <row r="20" s="5" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
-      <c r="A20" s="30">
-        <v>1</v>
-      </c>
-      <c r="B20" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" s="31" t="s">
+    <row r="20" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
+      <c r="A20" s="18"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="56">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="M20" s="57"/>
+      <c r="N20" s="56"/>
+      <c r="O20" s="25"/>
+      <c r="P20" s="56">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="Q20" s="25"/>
+      <c r="R20" s="25"/>
+      <c r="S20" s="25"/>
+    </row>
+    <row r="21" s="4" customFormat="1" ht="25" customHeight="1" spans="1:19">
+      <c r="A21" s="15" t="s">
         <v>52</v>
-      </c>
-      <c r="F20" s="32"/>
-      <c r="G20" s="32"/>
-      <c r="H20" s="33"/>
-      <c r="I20" s="32"/>
-      <c r="J20" s="59"/>
-      <c r="K20" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="L20" s="56" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M20" s="57" t="s">
-        <v>37</v>
-      </c>
-      <c r="N20" s="56" t="s">
-        <v>38</v>
-      </c>
-      <c r="O20" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="P20" s="56" t="e">
-        <f>N20+M20-O20</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q20" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="R20" s="25"/>
-      <c r="S20" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" s="4" customFormat="1" ht="23.25" customHeight="1" spans="1:19">
-      <c r="A21" s="15" t="s">
-        <v>53</v>
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="16"/>
       <c r="D21" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="28"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="58"/>
+      <c r="K21" s="23">
+        <f>SUM(K22:K22)</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="23" t="e">
+        <f>SUM(L22:L22)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M21" s="23">
+        <f t="shared" ref="M21:S21" si="15">SUM(M22:M22)</f>
+        <v>0</v>
+      </c>
+      <c r="N21" s="23">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="O21" s="23">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="P21" s="23" t="e">
+        <f t="shared" si="15"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q21" s="23">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="R21" s="23">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="S21" s="23"/>
+    </row>
+    <row r="22" s="5" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
+      <c r="A22" s="30">
+        <v>1</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="E21" s="23">
-        <f t="shared" ref="E21:J21" si="15">SUM(E22:E22)</f>
-        <v>0</v>
-      </c>
-      <c r="F21" s="23">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="G21" s="23">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="H21" s="23">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="I21" s="23">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="J21" s="23">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="K21" s="23">
-        <f ca="1" t="shared" ref="K21:R21" si="16">SUM(K23:K23)</f>
-        <v>0</v>
-      </c>
-      <c r="L21" s="23">
-        <f>SUM(L22:L22)</f>
-        <v>0</v>
-      </c>
-      <c r="M21" s="23">
-        <f ca="1" t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="N21" s="23">
-        <f ca="1" t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="O21" s="23">
-        <f ca="1" t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="P21" s="23">
-        <f>SUM(P22:P22)</f>
-        <v>0</v>
-      </c>
-      <c r="Q21" s="23">
-        <f ca="1" t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="R21" s="23">
-        <f ca="1" t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="S21" s="23"/>
-    </row>
-    <row r="22" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
-      <c r="A22" s="18"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="36"/>
-      <c r="J22" s="36"/>
-      <c r="K22" s="60"/>
-      <c r="L22" s="56">
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="33"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="59"/>
+      <c r="K22" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="L22" s="56" t="e">
         <f>E22+I22+J22</f>
-        <v>0</v>
-      </c>
-      <c r="M22" s="25"/>
-      <c r="N22" s="61"/>
-      <c r="O22" s="25"/>
-      <c r="P22" s="56">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M22" s="57" t="s">
+        <v>37</v>
+      </c>
+      <c r="N22" s="56" t="s">
+        <v>38</v>
+      </c>
+      <c r="O22" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="P22" s="56" t="e">
         <f>N22+M22-O22</f>
-        <v>0</v>
-      </c>
-      <c r="Q22" s="25"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q22" s="25" t="s">
+        <v>40</v>
+      </c>
       <c r="R22" s="25"/>
-      <c r="S22" s="25"/>
-    </row>
-    <row r="23" s="6" customFormat="1" ht="33" customHeight="1" spans="1:19">
-      <c r="A23" s="37" t="s">
+      <c r="S22" s="25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" s="4" customFormat="1" ht="23.25" customHeight="1" spans="1:19">
+      <c r="A23" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="41"/>
-      <c r="H23" s="41"/>
-      <c r="I23" s="41"/>
-      <c r="J23" s="62"/>
-      <c r="K23" s="63">
-        <f ca="1" t="shared" ref="K23:R23" si="17">K9+K11+K13+K15+K17+K19+K21</f>
-        <v>0</v>
-      </c>
-      <c r="L23" s="63" t="e">
-        <f t="shared" si="17"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="E23" s="23">
+        <f t="shared" ref="E23:J23" si="16">SUM(E24:E24)</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="23">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="G23" s="23">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="H23" s="23">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="I23" s="23">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="J23" s="23">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="K23" s="23">
+        <f ca="1" t="shared" ref="K23:R23" si="17">SUM(K25:K25)</f>
+        <v>0</v>
+      </c>
+      <c r="L23" s="23">
+        <f>SUM(L24:L24)</f>
+        <v>0</v>
+      </c>
+      <c r="M23" s="23">
+        <f ca="1" t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="N23" s="23">
+        <f ca="1" t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="O23" s="23">
+        <f ca="1" t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="P23" s="23">
+        <f>SUM(P24:P24)</f>
+        <v>0</v>
+      </c>
+      <c r="Q23" s="23">
+        <f ca="1" t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="R23" s="23">
+        <f ca="1" t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="S23" s="23"/>
+    </row>
+    <row r="24" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
+      <c r="A24" s="18"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="36"/>
+      <c r="J24" s="36"/>
+      <c r="K24" s="60"/>
+      <c r="L24" s="56">
+        <f>E24+I24+J24</f>
+        <v>0</v>
+      </c>
+      <c r="M24" s="25"/>
+      <c r="N24" s="61"/>
+      <c r="O24" s="25"/>
+      <c r="P24" s="56">
+        <f>N24+M24-O24</f>
+        <v>0</v>
+      </c>
+      <c r="Q24" s="25"/>
+      <c r="R24" s="25"/>
+      <c r="S24" s="25"/>
+    </row>
+    <row r="25" s="6" customFormat="1" ht="33" customHeight="1" spans="1:19">
+      <c r="A25" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" s="38"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="39"/>
+      <c r="E25" s="40"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="41"/>
+      <c r="H25" s="41"/>
+      <c r="I25" s="41"/>
+      <c r="J25" s="62"/>
+      <c r="K25" s="63">
+        <f ca="1" t="shared" ref="K25:R25" si="18">K9+K11+K13+K15+K17+K21+K23</f>
+        <v>0</v>
+      </c>
+      <c r="L25" s="63" t="e">
+        <f>L9+L11+L13+L15+L17+L21+L23</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M23" s="63">
-        <f ca="1" t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="N23" s="63">
-        <f ca="1" t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="O23" s="63">
-        <f ca="1" t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="P23" s="63" t="e">
-        <f t="shared" si="17"/>
+      <c r="M25" s="63">
+        <f ca="1" t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="N25" s="63">
+        <f ca="1" t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="O25" s="63">
+        <f ca="1" t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="P25" s="63" t="e">
+        <f t="shared" si="18"/>
         <v>#VALUE!</v>
       </c>
-      <c r="Q23" s="63">
-        <f ca="1" t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="R23" s="63">
-        <f ca="1" t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="S23" s="63"/>
-    </row>
-    <row r="24" s="6" customFormat="1" ht="33" customHeight="1" spans="3:19">
-      <c r="C24" s="42" t="s">
-        <v>56</v>
-      </c>
-      <c r="D24" s="42"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="42"/>
-      <c r="G24" s="42"/>
-      <c r="H24" s="43"/>
-      <c r="M24" s="64">
-        <f ca="1">N23</f>
-        <v>0</v>
-      </c>
-      <c r="N24" s="64"/>
-      <c r="O24" s="65"/>
-      <c r="P24" s="65"/>
-      <c r="Q24" s="68"/>
-      <c r="S24" s="68"/>
-    </row>
-    <row r="25" s="6" customFormat="1" ht="33" customHeight="1" spans="3:18">
-      <c r="C25" s="43" t="s">
-        <v>57</v>
-      </c>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="43"/>
-      <c r="M25" s="66">
-        <f ca="1">M24*10%</f>
-        <v>0</v>
-      </c>
-      <c r="N25" s="66"/>
-      <c r="O25" s="65"/>
-      <c r="P25" s="67"/>
-      <c r="Q25" s="67"/>
-      <c r="R25" s="68"/>
-    </row>
-    <row r="26" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
-      <c r="C26" s="43" t="s">
+      <c r="Q25" s="63">
+        <f ca="1" t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="R25" s="63">
+        <f ca="1" t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="S25" s="63"/>
+    </row>
+    <row r="26" s="6" customFormat="1" ht="33" customHeight="1" spans="3:19">
+      <c r="C26" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="D26" s="43"/>
-      <c r="E26" s="43"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="43"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="42"/>
+      <c r="F26" s="42"/>
+      <c r="G26" s="42"/>
       <c r="H26" s="43"/>
-      <c r="I26" s="68"/>
-      <c r="M26" s="66">
-        <f ca="1">M24-M25</f>
-        <v>0</v>
-      </c>
-      <c r="N26" s="66"/>
+      <c r="M26" s="64">
+        <f ca="1">N25</f>
+        <v>0</v>
+      </c>
+      <c r="N26" s="64"/>
       <c r="O26" s="65"/>
-      <c r="P26" s="67"/>
-      <c r="Q26" s="67"/>
-    </row>
-    <row r="27" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
-      <c r="C27" s="44" t="s">
+      <c r="P26" s="65"/>
+      <c r="Q26" s="68"/>
+      <c r="S26" s="68"/>
+    </row>
+    <row r="27" s="6" customFormat="1" ht="33" customHeight="1" spans="3:18">
+      <c r="C27" s="43" t="s">
         <v>59</v>
       </c>
-      <c r="D27" s="44"/>
-      <c r="E27" s="44"/>
-      <c r="F27" s="44"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="45"/>
-      <c r="I27" s="69"/>
-      <c r="J27" s="70"/>
-      <c r="K27" s="70"/>
-      <c r="L27" s="70"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="43"/>
       <c r="M27" s="66">
-        <f ca="1">R23-M26</f>
+        <f ca="1">M26*10%</f>
         <v>0</v>
       </c>
       <c r="N27" s="66"/>
       <c r="O27" s="65"/>
       <c r="P27" s="67"/>
       <c r="Q27" s="67"/>
-    </row>
-    <row r="28" s="7" customFormat="1" ht="33" customHeight="1" spans="1:18">
-      <c r="A28" s="46" t="s">
+      <c r="R27" s="68"/>
+    </row>
+    <row r="28" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
+      <c r="C28" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="B28" s="46"/>
-      <c r="C28" s="46"/>
-      <c r="D28" s="46"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="47"/>
-      <c r="G28" s="48"/>
-      <c r="H28" s="48"/>
-      <c r="I28" s="48"/>
-      <c r="J28" s="48"/>
-      <c r="M28" s="48"/>
-      <c r="N28" s="48"/>
-      <c r="O28" s="48"/>
-      <c r="P28" s="48"/>
-      <c r="Q28" s="48" t="s">
+      <c r="D28" s="43"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="43"/>
+      <c r="H28" s="43"/>
+      <c r="I28" s="68"/>
+      <c r="M28" s="66">
+        <f ca="1">M26-M27</f>
+        <v>0</v>
+      </c>
+      <c r="N28" s="66"/>
+      <c r="O28" s="65"/>
+      <c r="P28" s="67"/>
+      <c r="Q28" s="67"/>
+    </row>
+    <row r="29" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
+      <c r="C29" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="R28" s="48"/>
-    </row>
-    <row r="29" s="1" customFormat="1" ht="33" customHeight="1"/>
-    <row r="30" s="1" customFormat="1" ht="33" customHeight="1"/>
-    <row r="32" s="1" customFormat="1" spans="18:18">
-      <c r="R32" s="73"/>
-    </row>
-    <row r="35" s="1" customFormat="1" spans="1:18">
-      <c r="A35" s="48" t="s">
+      <c r="D29" s="44"/>
+      <c r="E29" s="44"/>
+      <c r="F29" s="44"/>
+      <c r="G29" s="44"/>
+      <c r="H29" s="45"/>
+      <c r="I29" s="69"/>
+      <c r="J29" s="70"/>
+      <c r="K29" s="70"/>
+      <c r="L29" s="70"/>
+      <c r="M29" s="66">
+        <f ca="1">R25-M28</f>
+        <v>0</v>
+      </c>
+      <c r="N29" s="66"/>
+      <c r="O29" s="65"/>
+      <c r="P29" s="67"/>
+      <c r="Q29" s="67"/>
+    </row>
+    <row r="30" s="7" customFormat="1" ht="33" customHeight="1" spans="1:18">
+      <c r="A30" s="46" t="s">
         <v>62</v>
       </c>
-      <c r="B35" s="48"/>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
-      <c r="G35" s="48"/>
-      <c r="H35" s="48"/>
-      <c r="I35" s="48"/>
-      <c r="J35" s="48"/>
-      <c r="K35" s="7"/>
-      <c r="M35" s="48"/>
-      <c r="N35" s="48"/>
-      <c r="O35" s="48"/>
-      <c r="P35" s="48"/>
-      <c r="Q35" s="48" t="s">
+      <c r="B30" s="46"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="47"/>
+      <c r="F30" s="47"/>
+      <c r="G30" s="48"/>
+      <c r="H30" s="48"/>
+      <c r="I30" s="48"/>
+      <c r="J30" s="48"/>
+      <c r="M30" s="48"/>
+      <c r="N30" s="48"/>
+      <c r="O30" s="48"/>
+      <c r="P30" s="48"/>
+      <c r="Q30" s="48" t="s">
         <v>63</v>
       </c>
-      <c r="R35" s="48"/>
-    </row>
-    <row r="36" s="4" customFormat="1" spans="3:14">
-      <c r="C36" s="49"/>
-      <c r="D36" s="49"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="49"/>
-      <c r="G36" s="49"/>
-      <c r="H36" s="49"/>
-      <c r="N36" s="65"/>
+      <c r="R30" s="48"/>
+    </row>
+    <row r="31" s="1" customFormat="1" ht="33" customHeight="1"/>
+    <row r="32" s="1" customFormat="1" ht="33" customHeight="1"/>
+    <row r="34" s="1" customFormat="1" spans="18:18">
+      <c r="R34" s="73"/>
+    </row>
+    <row r="37" s="1" customFormat="1" spans="1:18">
+      <c r="A37" s="48" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="48"/>
+      <c r="C37" s="48"/>
+      <c r="D37" s="48"/>
+      <c r="G37" s="48"/>
+      <c r="H37" s="48"/>
+      <c r="I37" s="48"/>
+      <c r="J37" s="48"/>
+      <c r="K37" s="7"/>
+      <c r="M37" s="48"/>
+      <c r="N37" s="48"/>
+      <c r="O37" s="48"/>
+      <c r="P37" s="48"/>
+      <c r="Q37" s="48" t="s">
+        <v>65</v>
+      </c>
+      <c r="R37" s="48"/>
+    </row>
+    <row r="38" s="4" customFormat="1" spans="3:14">
+      <c r="C38" s="49"/>
+      <c r="D38" s="49"/>
+      <c r="E38" s="49"/>
+      <c r="F38" s="49"/>
+      <c r="G38" s="49"/>
+      <c r="H38" s="49"/>
+      <c r="N38" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="23">
     <mergeCell ref="D1:F1"/>
-    <mergeCell ref="E19:J19"/>
-    <mergeCell ref="E20:J20"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="M25:N25"/>
-    <mergeCell ref="P25:Q25"/>
+    <mergeCell ref="E21:J21"/>
+    <mergeCell ref="E22:J22"/>
+    <mergeCell ref="A25:D25"/>
     <mergeCell ref="C26:G26"/>
     <mergeCell ref="M26:N26"/>
-    <mergeCell ref="P26:Q26"/>
     <mergeCell ref="C27:G27"/>
     <mergeCell ref="M27:N27"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="M28:O28"/>
-    <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="G35:J35"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="Q35:R35"/>
-    <mergeCell ref="C36:G36"/>
+    <mergeCell ref="P27:Q27"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="P28:Q28"/>
+    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="M30:O30"/>
+    <mergeCell ref="Q30:R30"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="G37:J37"/>
+    <mergeCell ref="M37:O37"/>
+    <mergeCell ref="Q37:R37"/>
+    <mergeCell ref="C38:G38"/>
   </mergeCells>
   <conditionalFormatting sqref="B4">
     <cfRule type="duplicateValues" dxfId="0" priority="10"/>
@@ -3034,19 +3134,19 @@
   <conditionalFormatting sqref="C17">
     <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C19">
+  <conditionalFormatting sqref="C21">
     <cfRule type="duplicateValues" dxfId="0" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C21">
+  <conditionalFormatting sqref="C23">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C7">
     <cfRule type="duplicateValues" dxfId="0" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C29:C34">
+  <conditionalFormatting sqref="C31:C36">
     <cfRule type="duplicateValues" dxfId="0" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1 C37:C1048576">
+  <conditionalFormatting sqref="C1 C39:C1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="11"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
cập nhật mẫu chi hoa hồng và thêm mẫu xuất hoá đơn
</commit_message>
<xml_diff>
--- a/public/templates/mau-chi-hoa-hong-text.xlsx
+++ b/public/templates/mau-chi-hoa-hong-text.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="10440"/>
+    <workbookView windowWidth="22188" windowHeight="10440"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>CÔNG TY TNHH HÓA ĐƠN ĐIỆN TỬ M-INVOICE - CHI NHÁNH TP. HỒ CHÍ MINH</t>
   </si>
@@ -119,42 +119,6 @@
     <t>TÊN CTY</t>
   </si>
   <si>
-    <t>BQ</t>
-  </si>
-  <si>
-    <t>SL MỚI</t>
-  </si>
-  <si>
-    <t>SL GH</t>
-  </si>
-  <si>
-    <t>SL TẶNG</t>
-  </si>
-  <si>
-    <t>GÓI HÓA ĐƠN</t>
-  </si>
-  <si>
-    <t>KHÁC</t>
-  </si>
-  <si>
-    <t>TỔNG XUẤT HĐ</t>
-  </si>
-  <si>
-    <t>VIẾT CHÊNH</t>
-  </si>
-  <si>
-    <t>HH</t>
-  </si>
-  <si>
-    <t>DT VIẾT CHÊNH</t>
-  </si>
-  <si>
-    <t>SỐ TIỀN</t>
-  </si>
-  <si>
-    <t>CHI CHÚ</t>
-  </si>
-  <si>
     <t>MTT</t>
   </si>
   <si>
@@ -189,9 +153,6 @@
   </si>
   <si>
     <t>G. GIÁ TRỊ CHỮ KÝ SỐ</t>
-  </si>
-  <si>
-    <t>TÊN SP</t>
   </si>
   <si>
     <t>KHAC</t>
@@ -2150,9 +2111,9 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L9" s="17" t="e">
+      <c r="L9" s="17">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="M9" s="17">
         <f t="shared" si="1"/>
@@ -2166,9 +2127,9 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P9" s="17" t="e">
+      <c r="P9" s="17">
         <f t="shared" si="1"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="17">
         <f t="shared" ref="Q9:Q13" si="3">SUM(Q10:Q10)</f>
@@ -2193,60 +2154,36 @@
       <c r="D10" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E10" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="F10" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="G10" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="H10" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="I10" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="J10" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="K10" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="L10" s="56" t="e">
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="56">
         <f t="shared" ref="L10:L14" si="5">E10+I10+J10</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M10" s="57" t="s">
-        <v>37</v>
-      </c>
-      <c r="N10" s="56" t="s">
-        <v>38</v>
-      </c>
-      <c r="O10" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="P10" s="56" t="e">
+        <v>0</v>
+      </c>
+      <c r="M10" s="57"/>
+      <c r="N10" s="56"/>
+      <c r="O10" s="25"/>
+      <c r="P10" s="56">
         <f t="shared" ref="P10:P14" si="6">N10+M10-O10</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q10" s="25" t="s">
-        <v>40</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q10" s="25"/>
       <c r="R10" s="25"/>
-      <c r="S10" s="25" t="s">
-        <v>41</v>
-      </c>
+      <c r="S10" s="25"/>
     </row>
     <row r="11" s="4" customFormat="1" ht="23.25" customHeight="1" spans="1:19">
       <c r="A11" s="15" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
       <c r="D11" s="15" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="E11" s="23">
         <f t="shared" si="0"/>
@@ -2304,7 +2241,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S11" s="23"/>
+      <c r="S11" s="17"/>
     </row>
     <row r="12" s="4" customFormat="1" ht="34.5" customHeight="1" spans="1:19">
       <c r="A12" s="18"/>
@@ -2335,12 +2272,12 @@
     </row>
     <row r="13" s="4" customFormat="1" ht="23.25" customHeight="1" spans="1:20">
       <c r="A13" s="15" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="D13" s="15" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E13" s="23">
         <f t="shared" si="0"/>
@@ -2398,7 +2335,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="S13" s="23"/>
+      <c r="S13" s="17"/>
       <c r="T13" s="72"/>
     </row>
     <row r="14" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
@@ -2430,12 +2367,12 @@
     </row>
     <row r="15" s="4" customFormat="1" ht="23.25" customHeight="1" spans="1:20">
       <c r="A15" s="15" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
       <c r="D15" s="15" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="E15" s="23">
         <f t="shared" ref="E15:O15" si="9">SUM(E16:E16)</f>
@@ -2482,7 +2419,7 @@
         <v>0</v>
       </c>
       <c r="P15" s="23">
-        <f t="shared" ref="P15:R15" si="10">SUM(P16:P16)</f>
+        <f t="shared" ref="P15:S15" si="10">SUM(P16:P16)</f>
         <v>0</v>
       </c>
       <c r="Q15" s="23">
@@ -2493,7 +2430,10 @@
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="S15" s="23"/>
+      <c r="S15" s="17">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
       <c r="T15" s="72"/>
     </row>
     <row r="16" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
@@ -2525,19 +2465,19 @@
     </row>
     <row r="17" s="4" customFormat="1" ht="23.25" customHeight="1" spans="1:20">
       <c r="A17" s="15" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="16"/>
       <c r="D17" s="15" t="s">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E17" s="23">
         <f>SUM(E18:E18)</f>
         <v>0</v>
       </c>
       <c r="F17" s="23">
-        <f t="shared" ref="E17:R17" si="13">SUM(F18:F18)</f>
+        <f t="shared" ref="E17:S17" si="13">SUM(F18:F18)</f>
         <v>0</v>
       </c>
       <c r="G17" s="23">
@@ -2588,7 +2528,7 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="S17" s="23"/>
+      <c r="S17" s="17"/>
       <c r="T17" s="72"/>
     </row>
     <row r="18" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
@@ -2620,15 +2560,15 @@
     </row>
     <row r="19" s="4" customFormat="1" ht="25" customHeight="1" spans="1:19">
       <c r="A19" s="15" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
       <c r="D19" s="15" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="E19" s="23">
-        <f t="shared" ref="E19:R19" si="14">SUM(E20:E20)</f>
+        <f t="shared" ref="E19:S19" si="14">SUM(E20:E20)</f>
         <v>0</v>
       </c>
       <c r="F19" s="23">
@@ -2683,7 +2623,7 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="S19" s="23"/>
+      <c r="S19" s="17"/>
     </row>
     <row r="20" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
       <c r="A20" s="18"/>
@@ -2714,12 +2654,12 @@
     </row>
     <row r="21" s="4" customFormat="1" ht="25" customHeight="1" spans="1:19">
       <c r="A21" s="15" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="16"/>
       <c r="D21" s="15" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="E21" s="28"/>
       <c r="F21" s="29"/>
@@ -2731,9 +2671,9 @@
         <f>SUM(K22:K22)</f>
         <v>0</v>
       </c>
-      <c r="L21" s="23" t="e">
+      <c r="L21" s="23">
         <f>SUM(L22:L22)</f>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="M21" s="23">
         <f t="shared" ref="M21:S21" si="15">SUM(M22:M22)</f>
@@ -2747,9 +2687,9 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="P21" s="23" t="e">
+      <c r="P21" s="23">
         <f t="shared" si="15"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="Q21" s="23">
         <f t="shared" si="15"/>
@@ -2759,65 +2699,45 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="S21" s="23"/>
+      <c r="S21" s="17"/>
     </row>
     <row r="22" s="5" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
       <c r="A22" s="30">
         <v>1</v>
       </c>
-      <c r="B22" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C22" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E22" s="31" t="s">
-        <v>54</v>
-      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="31"/>
       <c r="F22" s="32"/>
       <c r="G22" s="32"/>
       <c r="H22" s="33"/>
       <c r="I22" s="32"/>
       <c r="J22" s="59"/>
-      <c r="K22" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="L22" s="56" t="e">
+      <c r="K22" s="22"/>
+      <c r="L22" s="56">
         <f>E22+I22+J22</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M22" s="57" t="s">
-        <v>37</v>
-      </c>
-      <c r="N22" s="56" t="s">
-        <v>38</v>
-      </c>
-      <c r="O22" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="P22" s="56" t="e">
+        <v>0</v>
+      </c>
+      <c r="M22" s="57"/>
+      <c r="N22" s="56"/>
+      <c r="O22" s="25"/>
+      <c r="P22" s="56">
         <f>N22+M22-O22</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="Q22" s="25" t="s">
-        <v>40</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="25"/>
       <c r="R22" s="25"/>
-      <c r="S22" s="25" t="s">
-        <v>41</v>
-      </c>
+      <c r="S22" s="25"/>
     </row>
     <row r="23" s="4" customFormat="1" ht="23.25" customHeight="1" spans="1:19">
       <c r="A23" s="15" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="16"/>
       <c r="D23" s="15" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="E23" s="23">
         <f t="shared" ref="E23:J23" si="16">SUM(E24:E24)</f>
@@ -2875,7 +2795,7 @@
         <f ca="1" t="shared" si="17"/>
         <v>0</v>
       </c>
-      <c r="S23" s="23"/>
+      <c r="S23" s="17"/>
     </row>
     <row r="24" s="4" customFormat="1" ht="35.25" customHeight="1" spans="1:19">
       <c r="A24" s="18"/>
@@ -2906,7 +2826,7 @@
     </row>
     <row r="25" s="6" customFormat="1" ht="33" customHeight="1" spans="1:19">
       <c r="A25" s="37" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="B25" s="38"/>
       <c r="C25" s="38"/>
@@ -2918,12 +2838,12 @@
       <c r="I25" s="41"/>
       <c r="J25" s="62"/>
       <c r="K25" s="63">
-        <f ca="1" t="shared" ref="K25:R25" si="18">K9+K11+K13+K15+K17+K21+K23</f>
-        <v>0</v>
-      </c>
-      <c r="L25" s="63" t="e">
-        <f>L9+L11+L13+L15+L17+L21+L23</f>
-        <v>#VALUE!</v>
+        <f ca="1" t="shared" ref="K25:S25" si="18">K9+K11+K13+K15+K17+K21+K23</f>
+        <v>0</v>
+      </c>
+      <c r="L25" s="63">
+        <f t="shared" si="18"/>
+        <v>0</v>
       </c>
       <c r="M25" s="63">
         <f ca="1" t="shared" si="18"/>
@@ -2937,9 +2857,9 @@
         <f ca="1" t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="P25" s="63" t="e">
+      <c r="P25" s="63">
         <f t="shared" si="18"/>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="Q25" s="63">
         <f ca="1" t="shared" si="18"/>
@@ -2953,7 +2873,7 @@
     </row>
     <row r="26" s="6" customFormat="1" ht="33" customHeight="1" spans="3:19">
       <c r="C26" s="42" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D26" s="42"/>
       <c r="E26" s="42"/>
@@ -2972,7 +2892,7 @@
     </row>
     <row r="27" s="6" customFormat="1" ht="33" customHeight="1" spans="3:18">
       <c r="C27" s="43" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="D27" s="43"/>
       <c r="E27" s="43"/>
@@ -2991,7 +2911,7 @@
     </row>
     <row r="28" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
       <c r="C28" s="43" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="D28" s="43"/>
       <c r="E28" s="43"/>
@@ -3010,7 +2930,7 @@
     </row>
     <row r="29" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
       <c r="C29" s="44" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="D29" s="44"/>
       <c r="E29" s="44"/>
@@ -3032,7 +2952,7 @@
     </row>
     <row r="30" s="7" customFormat="1" ht="33" customHeight="1" spans="1:18">
       <c r="A30" s="46" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="B30" s="46"/>
       <c r="C30" s="46"/>
@@ -3048,7 +2968,7 @@
       <c r="O30" s="48"/>
       <c r="P30" s="48"/>
       <c r="Q30" s="48" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="R30" s="48"/>
     </row>
@@ -3059,7 +2979,7 @@
     </row>
     <row r="37" s="1" customFormat="1" spans="1:18">
       <c r="A37" s="48" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="B37" s="48"/>
       <c r="C37" s="48"/>
@@ -3074,7 +2994,7 @@
       <c r="O37" s="48"/>
       <c r="P37" s="48"/>
       <c r="Q37" s="48" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="R37" s="48"/>
     </row>

</xml_diff>

<commit_message>
chỉnh lại hàm delete,hiện error kĩ sản phẩm, chỉnh lại template mẫu đối soát
</commit_message>
<xml_diff>
--- a/public/templates/mau-chi-hoa-hong-text.xlsx
+++ b/public/templates/mau-chi-hoa-hong-text.xlsx
@@ -639,7 +639,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -710,30 +710,6 @@
         <color auto="1"/>
       </left>
       <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
       <top/>
       <bottom style="thin">
         <color auto="1"/>
@@ -796,19 +772,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -936,7 +899,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="14" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -948,34 +911,34 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="19" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1070,7 +1033,7 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1147,24 +1110,9 @@
     <xf numFmtId="58" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="5" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="6" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="6" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="8" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1172,19 +1120,19 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="182" fontId="1" fillId="0" borderId="3" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="8" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="182" fontId="10" fillId="3" borderId="3" xfId="56" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="57" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="57" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="57" applyFont="1" applyAlignment="1">
@@ -1216,10 +1164,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="51" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="12" xfId="53" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="10" xfId="53" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="182" fontId="1" fillId="0" borderId="3" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1229,13 +1177,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="182" fontId="1" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="51" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="13" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="3" fillId="5" borderId="10" xfId="51" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="183" fontId="3" fillId="5" borderId="8" xfId="51" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="184" fontId="3" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
@@ -1899,10 +1841,10 @@
       <c r="F3" s="10"/>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
-      <c r="M3" s="51"/>
-      <c r="N3" s="52"/>
-      <c r="O3" s="53"/>
-      <c r="P3" s="52"/>
+      <c r="M3" s="46"/>
+      <c r="N3" s="47"/>
+      <c r="O3" s="48"/>
+      <c r="P3" s="47"/>
     </row>
     <row r="4" s="2" customFormat="1" ht="28.9" customHeight="1" spans="2:19">
       <c r="B4" s="11"/>
@@ -1920,7 +1862,7 @@
       <c r="L4" s="11"/>
       <c r="M4" s="11"/>
       <c r="N4" s="11"/>
-      <c r="O4" s="54"/>
+      <c r="O4" s="49"/>
       <c r="P4" s="11"/>
       <c r="Q4" s="11"/>
       <c r="R4" s="11"/>
@@ -2007,7 +1949,7 @@
       <c r="N7" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="55" t="s">
+      <c r="O7" s="50" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2083,16 +2025,16 @@
         <f t="shared" ref="K9:K13" si="5">G9*85%</f>
         <v>0</v>
       </c>
-      <c r="L9" s="56">
+      <c r="L9" s="51">
         <f t="shared" ref="L9:L13" si="6">J9+K9</f>
         <v>0</v>
       </c>
-      <c r="M9" s="57"/>
-      <c r="N9" s="56">
+      <c r="M9" s="52"/>
+      <c r="N9" s="51">
         <f t="shared" ref="N9:N13" si="7">H9-M9</f>
         <v>0</v>
       </c>
-      <c r="O9" s="58"/>
+      <c r="O9" s="53"/>
     </row>
     <row r="10" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:15">
       <c r="A10" s="18" t="s">
@@ -2157,7 +2099,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I11" s="56"/>
+      <c r="I11" s="51"/>
       <c r="J11" s="25">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -2166,16 +2108,16 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L11" s="56">
+      <c r="L11" s="51">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="M11" s="58"/>
-      <c r="N11" s="56">
+      <c r="M11" s="53"/>
+      <c r="N11" s="51">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="O11" s="58"/>
+      <c r="O11" s="53"/>
     </row>
     <row r="12" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:16">
       <c r="A12" s="18" t="s">
@@ -2227,7 +2169,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="26"/>
-      <c r="P12" s="59"/>
+      <c r="P12" s="54"/>
     </row>
     <row r="13" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
       <c r="A13" s="21"/>
@@ -2241,7 +2183,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I13" s="58"/>
+      <c r="I13" s="53"/>
       <c r="J13" s="25">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -2250,16 +2192,16 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L13" s="56">
+      <c r="L13" s="51">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="M13" s="57"/>
-      <c r="N13" s="56">
+      <c r="M13" s="52"/>
+      <c r="N13" s="51">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="O13" s="58"/>
+      <c r="O13" s="53"/>
     </row>
     <row r="14" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:16">
       <c r="A14" s="18" t="s">
@@ -2311,7 +2253,7 @@
         <v>0</v>
       </c>
       <c r="O14" s="26"/>
-      <c r="P14" s="59"/>
+      <c r="P14" s="54"/>
     </row>
     <row r="15" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
       <c r="A15" s="21"/>
@@ -2334,16 +2276,16 @@
         <f t="shared" ref="K15:K19" si="13">G15*85%</f>
         <v>0</v>
       </c>
-      <c r="L15" s="56">
+      <c r="L15" s="51">
         <f t="shared" ref="L15:L19" si="14">J15+K15</f>
         <v>0</v>
       </c>
-      <c r="M15" s="57"/>
-      <c r="N15" s="56">
+      <c r="M15" s="52"/>
+      <c r="N15" s="51">
         <f t="shared" ref="N15:N19" si="15">H15-M15</f>
         <v>0</v>
       </c>
-      <c r="O15" s="58"/>
+      <c r="O15" s="53"/>
     </row>
     <row r="16" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:16">
       <c r="A16" s="18" t="s">
@@ -2395,7 +2337,7 @@
         <v>0</v>
       </c>
       <c r="O16" s="26"/>
-      <c r="P16" s="59"/>
+      <c r="P16" s="54"/>
     </row>
     <row r="17" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
       <c r="A17" s="21"/>
@@ -2418,16 +2360,16 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="L17" s="56">
+      <c r="L17" s="51">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="M17" s="57"/>
-      <c r="N17" s="56">
+      <c r="M17" s="52"/>
+      <c r="N17" s="51">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="O17" s="58"/>
+      <c r="O17" s="53"/>
     </row>
     <row r="18" s="3" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A18" s="18" t="s">
@@ -2501,16 +2443,16 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="L19" s="56">
+      <c r="L19" s="51">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="M19" s="57"/>
-      <c r="N19" s="56">
+      <c r="M19" s="52"/>
+      <c r="N19" s="51">
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="O19" s="58"/>
+      <c r="O19" s="53"/>
     </row>
     <row r="20" s="3" customFormat="1" ht="25" customHeight="1" spans="1:15">
       <c r="A20" s="18" t="s">
@@ -2521,12 +2463,30 @@
       <c r="D20" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="E20" s="30"/>
-      <c r="F20" s="31"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="31"/>
-      <c r="J20" s="60"/>
+      <c r="E20" s="26">
+        <f t="shared" ref="E20:J20" si="18">SUM(E21:E21)</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="26">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="G20" s="26">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="H20" s="26">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="I20" s="26">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="J20" s="26">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
       <c r="K20" s="26">
         <f>SUM(K21:K21)</f>
         <v>0</v>
@@ -2546,32 +2506,38 @@
       <c r="O20" s="26"/>
     </row>
     <row r="21" s="5" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
-      <c r="A21" s="32">
+      <c r="A21" s="30">
         <v>1</v>
       </c>
       <c r="B21" s="22"/>
       <c r="C21" s="23"/>
       <c r="D21" s="24"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="35"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="61"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25">
+        <f>F21+G21</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="25"/>
+      <c r="J21" s="25">
+        <f>I21*50%</f>
+        <v>0</v>
+      </c>
       <c r="K21" s="25">
         <f>G21*85%</f>
         <v>0</v>
       </c>
-      <c r="L21" s="56">
+      <c r="L21" s="51">
         <f>J21+K21</f>
         <v>0</v>
       </c>
-      <c r="M21" s="57"/>
-      <c r="N21" s="56">
+      <c r="M21" s="52"/>
+      <c r="N21" s="51">
         <f>H21-M21</f>
         <v>0</v>
       </c>
-      <c r="O21" s="58"/>
+      <c r="O21" s="53"/>
     </row>
     <row r="22" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:15">
       <c r="A22" s="18" t="s">
@@ -2583,27 +2549,27 @@
         <v>35</v>
       </c>
       <c r="E22" s="26">
-        <f t="shared" ref="E22:J22" si="18">SUM(E23:E23)</f>
+        <f t="shared" ref="E22:J22" si="19">SUM(E23:E23)</f>
         <v>0</v>
       </c>
       <c r="F22" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="G22" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="H22" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="I22" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="J22" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0</v>
       </c>
       <c r="K22" s="26">
@@ -2627,16 +2593,16 @@
     <row r="23" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
       <c r="A23" s="21"/>
       <c r="B23" s="22"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="38"/>
-      <c r="G23" s="38"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
       <c r="H23" s="25">
         <f>F23+G23</f>
         <v>0</v>
       </c>
-      <c r="I23" s="38"/>
+      <c r="I23" s="33"/>
       <c r="J23" s="25">
         <f>I23*50%</f>
         <v>0</v>
@@ -2645,200 +2611,198 @@
         <f>G23*85%</f>
         <v>0</v>
       </c>
-      <c r="L23" s="56">
+      <c r="L23" s="51">
         <f>J23+K23</f>
         <v>0</v>
       </c>
-      <c r="M23" s="58"/>
-      <c r="N23" s="56">
+      <c r="M23" s="53"/>
+      <c r="N23" s="51">
         <f>H23-M23</f>
         <v>0</v>
       </c>
-      <c r="O23" s="58"/>
+      <c r="O23" s="53"/>
     </row>
     <row r="24" s="6" customFormat="1" ht="33" customHeight="1" spans="1:15">
-      <c r="A24" s="39" t="s">
+      <c r="A24" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="40"/>
-      <c r="C24" s="40"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="42">
-        <f t="shared" ref="E24:O24" si="19">E8+E10+E12+E14+E16+E20+E22</f>
-        <v>0</v>
-      </c>
-      <c r="F24" s="42">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="G24" s="42">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="H24" s="42">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="I24" s="42">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="J24" s="42">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="K24" s="42">
-        <f ca="1" t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="L24" s="42">
-        <f t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="M24" s="42">
-        <f ca="1" t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="N24" s="42">
-        <f ca="1" t="shared" si="19"/>
-        <v>0</v>
-      </c>
-      <c r="O24" s="42"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="37">
+        <f t="shared" ref="E24:O24" si="20">E8+E10+E12+E14+E16+E20+E22</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="37">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="G24" s="37">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="H24" s="37">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="I24" s="37">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="J24" s="37">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="K24" s="37">
+        <f ca="1" t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="L24" s="37">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="M24" s="37">
+        <f ca="1" t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="N24" s="37">
+        <f ca="1" t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="O24" s="37"/>
     </row>
     <row r="25" s="6" customFormat="1" ht="33" customHeight="1" spans="3:18">
-      <c r="C25" s="43" t="s">
+      <c r="C25" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="D25" s="43"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
-      <c r="H25" s="44"/>
-      <c r="L25" s="62">
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="39"/>
+      <c r="L25" s="55">
         <f>L24</f>
         <v>0</v>
       </c>
       <c r="M25" s="3"/>
-      <c r="N25" s="63"/>
-      <c r="O25" s="63"/>
-      <c r="P25" s="64"/>
-      <c r="R25" s="66"/>
+      <c r="N25" s="56"/>
+      <c r="O25" s="56"/>
+      <c r="P25" s="57"/>
+      <c r="R25" s="59"/>
     </row>
     <row r="26" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
-      <c r="C26" s="44" t="s">
+      <c r="C26" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="D26" s="44"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="L26" s="65">
+      <c r="D26" s="39"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="39"/>
+      <c r="H26" s="39"/>
+      <c r="L26" s="58">
         <f>L25*10%</f>
         <v>0</v>
       </c>
       <c r="M26" s="3"/>
-      <c r="N26" s="63"/>
-      <c r="O26" s="63"/>
-      <c r="P26" s="63"/>
-      <c r="Q26" s="66"/>
+      <c r="N26" s="56"/>
+      <c r="O26" s="56"/>
+      <c r="P26" s="56"/>
+      <c r="Q26" s="59"/>
     </row>
     <row r="27" s="6" customFormat="1" ht="33" customHeight="1" spans="3:16">
-      <c r="C27" s="44" t="s">
+      <c r="C27" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="D27" s="44"/>
-      <c r="E27" s="44"/>
-      <c r="F27" s="44"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="44"/>
-      <c r="I27" s="66"/>
-      <c r="L27" s="65">
+      <c r="D27" s="39"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="39"/>
+      <c r="H27" s="39"/>
+      <c r="I27" s="59"/>
+      <c r="L27" s="58">
         <f>L25-L26</f>
         <v>0</v>
       </c>
-      <c r="N27" s="63"/>
-      <c r="O27" s="63"/>
-      <c r="P27" s="63"/>
+      <c r="N27" s="56"/>
+      <c r="O27" s="56"/>
+      <c r="P27" s="56"/>
     </row>
     <row r="28" s="6" customFormat="1" ht="33" customHeight="1" spans="3:16">
-      <c r="C28" s="45" t="s">
+      <c r="C28" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="D28" s="45"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="45"/>
-      <c r="G28" s="45"/>
-      <c r="H28" s="46"/>
-      <c r="I28" s="67"/>
-      <c r="J28" s="68"/>
-      <c r="K28" s="68"/>
-      <c r="L28" s="65">
+      <c r="D28" s="40"/>
+      <c r="E28" s="40"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="41"/>
+      <c r="I28" s="60"/>
+      <c r="J28" s="61"/>
+      <c r="K28" s="61"/>
+      <c r="L28" s="58">
         <f ca="1">H24-L24-M24</f>
         <v>0</v>
       </c>
-      <c r="N28" s="63"/>
-      <c r="O28" s="63"/>
-      <c r="P28" s="63"/>
+      <c r="N28" s="56"/>
+      <c r="O28" s="56"/>
+      <c r="P28" s="56"/>
     </row>
     <row r="29" s="7" customFormat="1" ht="33" customHeight="1" spans="1:16">
-      <c r="A29" s="47" t="s">
+      <c r="A29" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="B29" s="47"/>
-      <c r="C29" s="47"/>
-      <c r="D29" s="47"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="48"/>
-      <c r="G29" s="49"/>
-      <c r="H29" s="49"/>
-      <c r="I29" s="49"/>
-      <c r="J29" s="49"/>
-      <c r="M29" s="66"/>
-      <c r="N29" s="49" t="s">
+      <c r="B29" s="42"/>
+      <c r="C29" s="42"/>
+      <c r="D29" s="42"/>
+      <c r="E29" s="43"/>
+      <c r="F29" s="43"/>
+      <c r="G29" s="44"/>
+      <c r="H29" s="44"/>
+      <c r="I29" s="44"/>
+      <c r="J29" s="44"/>
+      <c r="M29" s="59"/>
+      <c r="N29" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="O29" s="49"/>
-      <c r="P29" s="69"/>
+      <c r="O29" s="44"/>
+      <c r="P29" s="62"/>
     </row>
     <row r="30" s="1" customFormat="1" ht="33" customHeight="1"/>
     <row r="31" s="1" customFormat="1" ht="63" customHeight="1"/>
     <row r="32" spans="1:15">
-      <c r="A32" s="49" t="s">
+      <c r="A32" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="B32" s="49"/>
-      <c r="C32" s="49"/>
-      <c r="D32" s="49"/>
-      <c r="N32" s="49" t="s">
+      <c r="B32" s="44"/>
+      <c r="C32" s="44"/>
+      <c r="D32" s="44"/>
+      <c r="N32" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="O32" s="49"/>
+      <c r="O32" s="44"/>
     </row>
     <row r="33" s="1" customFormat="1" spans="18:18">
-      <c r="R33" s="71"/>
+      <c r="R33" s="64"/>
     </row>
     <row r="36" s="1" customFormat="1" spans="7:11">
-      <c r="G36" s="49"/>
-      <c r="H36" s="49"/>
-      <c r="I36" s="49"/>
-      <c r="J36" s="49"/>
+      <c r="G36" s="44"/>
+      <c r="H36" s="44"/>
+      <c r="I36" s="44"/>
+      <c r="J36" s="44"/>
       <c r="K36" s="7"/>
     </row>
     <row r="37" s="3" customFormat="1" spans="3:14">
-      <c r="C37" s="50"/>
-      <c r="D37" s="50"/>
-      <c r="E37" s="50"/>
-      <c r="F37" s="50"/>
-      <c r="G37" s="50"/>
-      <c r="H37" s="50"/>
-      <c r="N37" s="70"/>
+      <c r="C37" s="45"/>
+      <c r="D37" s="45"/>
+      <c r="E37" s="45"/>
+      <c r="F37" s="45"/>
+      <c r="G37" s="45"/>
+      <c r="H37" s="45"/>
+      <c r="N37" s="63"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="13">
     <mergeCell ref="D1:F1"/>
-    <mergeCell ref="E20:J20"/>
-    <mergeCell ref="E21:J21"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="C25:G25"/>
     <mergeCell ref="C26:G26"/>

</xml_diff>

<commit_message>
sửa lại bộ lọc, chỉnh mẫu đối soát
</commit_message>
<xml_diff>
--- a/public/templates/mau-chi-hoa-hong-text.xlsx
+++ b/public/templates/mau-chi-hoa-hong-text.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>CÔNG TY TNHH HÓA ĐƠN ĐIỆN TỬ M-INVOICE - CHI NHÁNH TP. HỒ CHÍ MINH</t>
   </si>
@@ -59,16 +59,13 @@
     <t>SỐ LƯỢNG</t>
   </si>
   <si>
-    <t>DOANH THU SẢN PHẨM</t>
-  </si>
-  <si>
-    <t>PHÍ VIẾT CHÊNH</t>
-  </si>
-  <si>
     <t>GIÁ TRỊ XUẤT HÓA ĐƠN</t>
   </si>
   <si>
     <t xml:space="preserve">GIÁ ĐỐI SOÁT </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> GIÁ TRỊ VIẾT CHÊNH</t>
   </si>
   <si>
     <t>TIỀN HOA HỒNG</t>
@@ -639,7 +636,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -693,7 +690,9 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -753,21 +752,6 @@
         <color rgb="FF000000"/>
       </right>
       <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
@@ -899,7 +883,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -911,34 +895,34 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1033,7 +1017,7 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1104,6 +1088,9 @@
     <xf numFmtId="3" fontId="9" fillId="0" borderId="4" xfId="53" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="182" fontId="1" fillId="0" borderId="3" xfId="54" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="58" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1138,12 +1125,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="57" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="182" fontId="3" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="57" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="57" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="182" fontId="3" fillId="5" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="51" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1167,13 +1157,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="10" xfId="53" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="182" fontId="1" fillId="0" borderId="3" xfId="55" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="3" xfId="54" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="182" fontId="1" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1"/>
@@ -1183,9 +1167,6 @@
     <xf numFmtId="184" fontId="3" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="182" fontId="3" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="183" fontId="3" fillId="5" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="182" fontId="3" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="182" fontId="3" fillId="5" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="51" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="184" fontId="3" fillId="0" borderId="0" xfId="51" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="58" applyFont="1" applyFill="1"/>
@@ -1785,7 +1766,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S37"/>
+  <dimension ref="A1:R37"/>
   <sheetFormatPr defaultColWidth="7.71296296296296" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="5.28703703703704" style="1" customWidth="1"/>
@@ -1793,32 +1774,29 @@
     <col min="3" max="3" width="15.712962962963" style="1" customWidth="1"/>
     <col min="4" max="4" width="40.4259259259259" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.287037037037" style="1" customWidth="1"/>
-    <col min="6" max="6" width="11" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5740740740741" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.3611111111111" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5740740740741" style="1" customWidth="1"/>
-    <col min="10" max="10" width="10.4259259259259" style="1" customWidth="1"/>
-    <col min="11" max="11" width="12.712962962963" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15" style="1" customWidth="1"/>
-    <col min="13" max="13" width="10.4259259259259" style="1" customWidth="1"/>
-    <col min="14" max="14" width="11.712962962963" style="1" customWidth="1"/>
-    <col min="15" max="15" width="13.5092592592593" style="1" customWidth="1"/>
-    <col min="16" max="16" width="13.712962962963" style="1" customWidth="1"/>
-    <col min="17" max="17" width="12.287037037037" style="1" customWidth="1"/>
-    <col min="18" max="18" width="14.287037037037" style="1" customWidth="1"/>
-    <col min="19" max="19" width="9.57407407407407" style="1" customWidth="1"/>
-    <col min="20" max="20" width="9.42592592592593" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="7.71296296296296" style="1"/>
+    <col min="6" max="6" width="13.3611111111111" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.5740740740741" style="1" customWidth="1"/>
+    <col min="8" max="9" width="10.4259259259259" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.712962962963" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15" style="1" customWidth="1"/>
+    <col min="12" max="12" width="10.4259259259259" style="1" customWidth="1"/>
+    <col min="13" max="13" width="11.712962962963" style="1" customWidth="1"/>
+    <col min="14" max="14" width="13.5092592592593" style="1" customWidth="1"/>
+    <col min="15" max="15" width="13.712962962963" style="1" customWidth="1"/>
+    <col min="16" max="16" width="12.287037037037" style="1" customWidth="1"/>
+    <col min="17" max="17" width="14.287037037037" style="1" customWidth="1"/>
+    <col min="18" max="18" width="9.57407407407407" style="1" customWidth="1"/>
+    <col min="19" max="19" width="9.42592592592593" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="7.71296296296296" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.15" customHeight="1" spans="4:6">
+    <row r="1" s="1" customFormat="1" ht="28.15" customHeight="1" spans="4:5">
       <c r="D1" s="8" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-    </row>
-    <row r="2" s="1" customFormat="1" ht="13.8" spans="1:8">
+    </row>
+    <row r="2" s="1" customFormat="1" ht="13.8" spans="1:6">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -1826,11 +1804,9 @@
         <v>1</v>
       </c>
       <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-    </row>
-    <row r="3" s="1" customFormat="1" ht="13.8" spans="1:16">
+      <c r="F2" s="7"/>
+    </row>
+    <row r="3" s="1" customFormat="1" ht="13.8" spans="1:15">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -1838,46 +1814,44 @@
         <v>2</v>
       </c>
       <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="M3" s="46"/>
-      <c r="N3" s="47"/>
-      <c r="O3" s="48"/>
-      <c r="P3" s="47"/>
-    </row>
-    <row r="4" s="2" customFormat="1" ht="28.9" customHeight="1" spans="2:19">
+      <c r="F3" s="7"/>
+      <c r="L3" s="50"/>
+      <c r="M3" s="51"/>
+      <c r="N3" s="52"/>
+      <c r="O3" s="51"/>
+    </row>
+    <row r="4" s="2" customFormat="1" ht="28.9" customHeight="1" spans="2:18">
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
+      <c r="F4" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="G4" s="11"/>
-      <c r="H4" s="11" t="s">
-        <v>3</v>
-      </c>
+      <c r="H4" s="11"/>
       <c r="I4" s="11"/>
       <c r="J4" s="11"/>
       <c r="K4" s="11"/>
       <c r="L4" s="11"/>
       <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="49"/>
+      <c r="N4" s="53"/>
+      <c r="O4" s="11"/>
       <c r="P4" s="11"/>
       <c r="Q4" s="11"/>
       <c r="R4" s="11"/>
-      <c r="S4" s="11"/>
-    </row>
-    <row r="5" s="3" customFormat="1" ht="28.9" customHeight="1" spans="2:18">
+    </row>
+    <row r="5" s="3" customFormat="1" ht="28.9" customHeight="1" spans="2:17">
       <c r="B5" s="12"/>
       <c r="C5" s="12"/>
       <c r="D5" s="12"/>
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
+      <c r="G5" s="12" t="s">
+        <v>4</v>
+      </c>
       <c r="H5" s="12"/>
-      <c r="I5" s="12" t="s">
-        <v>4</v>
-      </c>
+      <c r="I5" s="12"/>
       <c r="J5" s="12"/>
       <c r="K5" s="12"/>
       <c r="L5" s="12"/>
@@ -1886,14 +1860,14 @@
       <c r="O5" s="12"/>
       <c r="P5" s="12"/>
       <c r="Q5" s="12"/>
-      <c r="R5" s="12"/>
-    </row>
-    <row r="6" s="3" customFormat="1" ht="18.15" spans="2:18">
+    </row>
+    <row r="6" s="3" customFormat="1" ht="18.15" spans="2:17">
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
       <c r="D6" s="12"/>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
       <c r="J6" s="12"/>
@@ -1904,9 +1878,8 @@
       <c r="O6" s="12"/>
       <c r="P6" s="12"/>
       <c r="Q6" s="12"/>
-      <c r="R6" s="12"/>
-    </row>
-    <row r="7" s="4" customFormat="1" ht="51" customHeight="1" spans="1:15">
+    </row>
+    <row r="7" s="4" customFormat="1" ht="51" customHeight="1" spans="1:14">
       <c r="A7" s="13" t="s">
         <v>5</v>
       </c>
@@ -1922,13 +1895,13 @@
       <c r="E7" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="17" t="s">
+      <c r="H7" s="16" t="s">
         <v>12</v>
       </c>
       <c r="I7" s="17" t="s">
@@ -1946,65 +1919,58 @@
       <c r="M7" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="N7" s="17" t="s">
+      <c r="N7" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="50" t="s">
+    </row>
+    <row r="8" s="3" customFormat="1" ht="29.25" customHeight="1" spans="1:14">
+      <c r="A8" s="18" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="8" s="3" customFormat="1" ht="29.25" customHeight="1" spans="1:15">
-      <c r="A8" s="18" t="s">
-        <v>20</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="19"/>
       <c r="D8" s="18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" s="20">
         <f t="shared" ref="E8:E12" si="0">SUM(E9:E9)</f>
         <v>0</v>
       </c>
       <c r="F8" s="20">
-        <f t="shared" ref="F8:P8" si="1">SUM(F9:F9)</f>
+        <f>SUM(F9:F9)</f>
         <v>0</v>
       </c>
       <c r="G8" s="20">
-        <f t="shared" ref="G8:G12" si="2">SUM(G9:G9)</f>
+        <f>SUM(G9:G9)</f>
         <v>0</v>
       </c>
       <c r="H8" s="20">
-        <f>SUM(H9:H9)</f>
+        <f t="shared" ref="H8:H12" si="1">SUM(H9:H9)</f>
         <v>0</v>
       </c>
       <c r="I8" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="I8:O8" si="2">SUM(I9:I9)</f>
         <v>0</v>
       </c>
       <c r="J8" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="K8" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L8" s="20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="M8" s="20">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N8" s="20">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O8" s="20"/>
-    </row>
-    <row r="9" s="3" customFormat="1" ht="34.5" customHeight="1" spans="1:15">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="N8" s="20"/>
+    </row>
+    <row r="9" s="3" customFormat="1" ht="34.5" customHeight="1" spans="1:14">
       <c r="A9" s="21"/>
       <c r="B9" s="22"/>
       <c r="C9" s="23"/>
@@ -2013,81 +1979,73 @@
       <c r="F9" s="25"/>
       <c r="G9" s="25"/>
       <c r="H9" s="25">
-        <f t="shared" ref="H9:H13" si="3">F9+G9</f>
+        <f>F9-G9</f>
         <v>0</v>
       </c>
       <c r="I9" s="25"/>
       <c r="J9" s="25">
-        <f t="shared" ref="J9:J13" si="4">I9*50%</f>
-        <v>0</v>
-      </c>
-      <c r="K9" s="25">
-        <f t="shared" ref="K9:K13" si="5">G9*85%</f>
-        <v>0</v>
-      </c>
-      <c r="L9" s="51">
-        <f t="shared" ref="L9:L13" si="6">J9+K9</f>
-        <v>0</v>
-      </c>
-      <c r="M9" s="52"/>
-      <c r="N9" s="51">
-        <f t="shared" ref="N9:N13" si="7">H9-M9</f>
-        <v>0</v>
-      </c>
-      <c r="O9" s="53"/>
-    </row>
-    <row r="10" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:15">
+        <f t="shared" ref="J9:J13" si="3">H9*85%</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="27">
+        <f t="shared" ref="K9:K13" si="4">I9+J9</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="55"/>
+      <c r="M9" s="27">
+        <f t="shared" ref="M9:M13" si="5">F9-L9</f>
+        <v>0</v>
+      </c>
+      <c r="N9" s="28"/>
+    </row>
+    <row r="10" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:14">
       <c r="A10" s="18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10" s="19"/>
       <c r="C10" s="19"/>
       <c r="D10" s="18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E10" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F10" s="26">
-        <f t="shared" ref="F10:P10" si="8">SUM(F11:F11)</f>
+        <f>SUM(F11:F11)</f>
         <v>0</v>
       </c>
       <c r="G10" s="26">
-        <f t="shared" si="2"/>
+        <f>SUM(G11:G11)</f>
         <v>0</v>
       </c>
       <c r="H10" s="26">
-        <f>SUM(H11:H11)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I10" s="26">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="I10:O10" si="6">SUM(I11:I11)</f>
         <v>0</v>
       </c>
       <c r="J10" s="26">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="K10" s="26">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L10" s="26">
-        <f t="shared" si="8"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="M10" s="26">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="N10" s="26">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="O10" s="26"/>
-    </row>
-    <row r="11" s="3" customFormat="1" ht="34.5" customHeight="1" spans="1:15">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="N10" s="26"/>
+    </row>
+    <row r="11" s="3" customFormat="1" ht="34.5" customHeight="1" spans="1:14">
       <c r="A11" s="21"/>
       <c r="B11" s="22"/>
       <c r="C11" s="23"/>
@@ -2096,417 +2054,377 @@
       <c r="F11" s="25"/>
       <c r="G11" s="27"/>
       <c r="H11" s="25">
+        <f t="shared" ref="H9:H13" si="7">F11-G11</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="25"/>
+      <c r="J11" s="25">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I11" s="51"/>
-      <c r="J11" s="25">
+      <c r="K11" s="27">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="K11" s="25">
+      <c r="L11" s="28"/>
+      <c r="M11" s="27">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L11" s="51">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="M11" s="53"/>
-      <c r="N11" s="51">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="O11" s="53"/>
-    </row>
-    <row r="12" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:16">
+      <c r="N11" s="28"/>
+    </row>
+    <row r="12" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:15">
       <c r="A12" s="18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12" s="19"/>
       <c r="C12" s="19"/>
       <c r="D12" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E12" s="26">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F12" s="26">
-        <f t="shared" ref="F12:P12" si="9">SUM(F13:F13)</f>
+        <f>SUM(F13:F13)</f>
         <v>0</v>
       </c>
       <c r="G12" s="26">
-        <f t="shared" si="2"/>
+        <f>SUM(G13:G13)</f>
         <v>0</v>
       </c>
       <c r="H12" s="26">
-        <f t="shared" si="9"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I12" s="26">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="I12:O12" si="8">SUM(I13:I13)</f>
         <v>0</v>
       </c>
       <c r="J12" s="26">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="K12" s="26">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="L12" s="26">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="M12" s="26">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="N12" s="26">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="O12" s="26"/>
-      <c r="P12" s="54"/>
-    </row>
-    <row r="13" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="N12" s="26"/>
+      <c r="O12" s="56"/>
+    </row>
+    <row r="13" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:14">
       <c r="A13" s="21"/>
       <c r="B13" s="22"/>
       <c r="C13" s="23"/>
       <c r="D13" s="24"/>
       <c r="E13" s="25"/>
       <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
+      <c r="G13" s="28"/>
       <c r="H13" s="25">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="I13" s="25"/>
+      <c r="J13" s="25">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I13" s="53"/>
-      <c r="J13" s="25">
+      <c r="K13" s="27">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="K13" s="25">
+      <c r="L13" s="55"/>
+      <c r="M13" s="27">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L13" s="51">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="M13" s="52"/>
-      <c r="N13" s="51">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="O13" s="53"/>
-    </row>
-    <row r="14" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:16">
+      <c r="N13" s="28"/>
+    </row>
+    <row r="14" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:15">
       <c r="A14" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B14" s="19"/>
       <c r="C14" s="19"/>
       <c r="D14" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E14" s="26">
-        <f t="shared" ref="E14:O14" si="10">SUM(E15:E15)</f>
+        <f>SUM(E15:E15)</f>
         <v>0</v>
       </c>
       <c r="F14" s="26">
-        <f t="shared" si="10"/>
+        <f>SUM(F15:F15)</f>
         <v>0</v>
       </c>
       <c r="G14" s="26">
-        <f t="shared" si="10"/>
+        <f>SUM(G15:G15)</f>
         <v>0</v>
       </c>
       <c r="H14" s="26">
-        <f t="shared" si="10"/>
+        <f>SUM(H15:H15)</f>
         <v>0</v>
       </c>
       <c r="I14" s="26">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="I14:N14" si="9">SUM(I15:I15)</f>
         <v>0</v>
       </c>
       <c r="J14" s="26">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="K14" s="26">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="L14" s="26">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="M14" s="26">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="N14" s="26">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="O14" s="26"/>
-      <c r="P14" s="54"/>
-    </row>
-    <row r="15" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="N14" s="26"/>
+      <c r="O14" s="56"/>
+    </row>
+    <row r="15" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:14">
       <c r="A15" s="21"/>
       <c r="B15" s="22"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="30"/>
       <c r="E15" s="25"/>
       <c r="F15" s="25"/>
       <c r="G15" s="25"/>
       <c r="H15" s="25">
-        <f t="shared" ref="H15:H19" si="11">F15+G15</f>
+        <f t="shared" ref="H15:H19" si="10">F15-G15</f>
         <v>0</v>
       </c>
       <c r="I15" s="25"/>
       <c r="J15" s="25">
-        <f t="shared" ref="J15:J19" si="12">I15*50%</f>
-        <v>0</v>
-      </c>
-      <c r="K15" s="25">
-        <f t="shared" ref="K15:K19" si="13">G15*85%</f>
-        <v>0</v>
-      </c>
-      <c r="L15" s="51">
-        <f t="shared" ref="L15:L19" si="14">J15+K15</f>
-        <v>0</v>
-      </c>
-      <c r="M15" s="52"/>
-      <c r="N15" s="51">
-        <f t="shared" ref="N15:N19" si="15">H15-M15</f>
-        <v>0</v>
-      </c>
-      <c r="O15" s="53"/>
-    </row>
-    <row r="16" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:16">
+        <f t="shared" ref="J15:J19" si="11">H15*85%</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="27">
+        <f t="shared" ref="K15:K19" si="12">I15+J15</f>
+        <v>0</v>
+      </c>
+      <c r="L15" s="55"/>
+      <c r="M15" s="27">
+        <f t="shared" ref="M15:M19" si="13">F15-L15</f>
+        <v>0</v>
+      </c>
+      <c r="N15" s="28"/>
+    </row>
+    <row r="16" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:15">
       <c r="A16" s="18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" s="19"/>
       <c r="C16" s="19"/>
       <c r="D16" s="18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E16" s="26">
         <f>SUM(E17:E17)</f>
         <v>0</v>
       </c>
       <c r="F16" s="26">
-        <f t="shared" ref="E16:S16" si="16">SUM(F17:F17)</f>
+        <f>SUM(F17:F17)</f>
         <v>0</v>
       </c>
       <c r="G16" s="26">
-        <f t="shared" si="16"/>
+        <f>SUM(G17:G17)</f>
         <v>0</v>
       </c>
       <c r="H16" s="26">
-        <f t="shared" si="16"/>
+        <f>SUM(H17:H17)</f>
         <v>0</v>
       </c>
       <c r="I16" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" ref="I16:R16" si="14">SUM(I17:I17)</f>
         <v>0</v>
       </c>
       <c r="J16" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="K16" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="L16" s="26">
-        <f t="shared" si="16"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="M16" s="26">
-        <f t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="N16" s="26">
-        <f t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="O16" s="26"/>
-      <c r="P16" s="54"/>
-    </row>
-    <row r="17" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="N16" s="26"/>
+      <c r="O16" s="56"/>
+    </row>
+    <row r="17" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:14">
       <c r="A17" s="21"/>
       <c r="B17" s="22"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="29"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="30"/>
       <c r="E17" s="25"/>
       <c r="F17" s="25"/>
       <c r="G17" s="25"/>
       <c r="H17" s="25">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="I17" s="25"/>
       <c r="J17" s="25">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="K17" s="27">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="K17" s="25">
+      <c r="L17" s="55"/>
+      <c r="M17" s="27">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="L17" s="51">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="M17" s="52"/>
-      <c r="N17" s="51">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="O17" s="53"/>
-    </row>
-    <row r="18" s="3" customFormat="1" ht="25" customHeight="1" spans="1:15">
+      <c r="N17" s="28"/>
+    </row>
+    <row r="18" s="3" customFormat="1" ht="25" customHeight="1" spans="1:14">
       <c r="A18" s="18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18" s="19"/>
       <c r="C18" s="19"/>
       <c r="D18" s="18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E18" s="26">
-        <f t="shared" ref="E18:S18" si="17">SUM(E19:E19)</f>
+        <f>SUM(E19:E19)</f>
         <v>0</v>
       </c>
       <c r="F18" s="26">
-        <f t="shared" si="17"/>
+        <f>SUM(F19:F19)</f>
         <v>0</v>
       </c>
       <c r="G18" s="26">
-        <f t="shared" si="17"/>
+        <f>SUM(G19:G19)</f>
         <v>0</v>
       </c>
       <c r="H18" s="26">
-        <f t="shared" si="17"/>
+        <f>SUM(H19:H19)</f>
         <v>0</v>
       </c>
       <c r="I18" s="26">
-        <f t="shared" si="17"/>
+        <f t="shared" ref="I18:R18" si="15">SUM(I19:I19)</f>
         <v>0</v>
       </c>
       <c r="J18" s="26">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="K18" s="26">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="L18" s="26">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="M18" s="26">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="N18" s="26">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
-      <c r="O18" s="26"/>
-    </row>
-    <row r="19" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="N18" s="26"/>
+    </row>
+    <row r="19" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:14">
       <c r="A19" s="21"/>
       <c r="B19" s="22"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="30"/>
       <c r="E19" s="25"/>
       <c r="F19" s="25"/>
       <c r="G19" s="25"/>
       <c r="H19" s="25">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="I19" s="25"/>
       <c r="J19" s="25">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="K19" s="27">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="K19" s="25">
+      <c r="L19" s="55"/>
+      <c r="M19" s="27">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="L19" s="51">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="M19" s="52"/>
-      <c r="N19" s="51">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="O19" s="53"/>
-    </row>
-    <row r="20" s="3" customFormat="1" ht="25" customHeight="1" spans="1:15">
+      <c r="N19" s="28"/>
+    </row>
+    <row r="20" s="3" customFormat="1" ht="25" customHeight="1" spans="1:14">
       <c r="A20" s="18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B20" s="19"/>
       <c r="C20" s="19"/>
       <c r="D20" s="18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" s="26">
-        <f t="shared" ref="E20:J20" si="18">SUM(E21:E21)</f>
+        <f>SUM(E21:E21)</f>
         <v>0</v>
       </c>
       <c r="F20" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" ref="F20:M20" si="16">SUM(F21:F21)</f>
         <v>0</v>
       </c>
       <c r="G20" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="H20" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="I20" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="J20" s="26">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="K20" s="26">
-        <f>SUM(K21:K21)</f>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="L20" s="26">
-        <f>SUM(L21:L21)</f>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="M20" s="26">
-        <f>SUM(M21:M21)</f>
-        <v>0</v>
-      </c>
-      <c r="N20" s="26">
-        <f>SUM(N21:N21)</f>
-        <v>0</v>
-      </c>
-      <c r="O20" s="26"/>
-    </row>
-    <row r="21" s="5" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
-      <c r="A21" s="30">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="N20" s="26"/>
+    </row>
+    <row r="21" s="5" customFormat="1" ht="35.25" customHeight="1" spans="1:14">
+      <c r="A21" s="31">
         <v>1</v>
       </c>
       <c r="B21" s="22"/>
@@ -2516,305 +2434,279 @@
       <c r="F21" s="25"/>
       <c r="G21" s="25"/>
       <c r="H21" s="25">
-        <f>F21+G21</f>
+        <f>F21-G21</f>
         <v>0</v>
       </c>
       <c r="I21" s="25"/>
       <c r="J21" s="25">
-        <f>I21*50%</f>
-        <v>0</v>
-      </c>
-      <c r="K21" s="25">
-        <f>G21*85%</f>
-        <v>0</v>
-      </c>
-      <c r="L21" s="51">
-        <f>J21+K21</f>
-        <v>0</v>
-      </c>
-      <c r="M21" s="52"/>
-      <c r="N21" s="51">
-        <f>H21-M21</f>
-        <v>0</v>
-      </c>
-      <c r="O21" s="53"/>
-    </row>
-    <row r="22" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:15">
+        <f>H21*85%</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="27">
+        <f>I21+J21</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="55"/>
+      <c r="M21" s="27">
+        <f>F21-L21</f>
+        <v>0</v>
+      </c>
+      <c r="N21" s="28"/>
+    </row>
+    <row r="22" s="3" customFormat="1" ht="23.25" customHeight="1" spans="1:14">
       <c r="A22" s="18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B22" s="19"/>
       <c r="C22" s="19"/>
       <c r="D22" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E22" s="26">
-        <f t="shared" ref="E22:J22" si="19">SUM(E23:E23)</f>
+        <f>SUM(E23:E23)</f>
         <v>0</v>
       </c>
       <c r="F22" s="26">
-        <f t="shared" si="19"/>
+        <f>SUM(F23:F23)</f>
         <v>0</v>
       </c>
       <c r="G22" s="26">
-        <f t="shared" si="19"/>
+        <f>SUM(G23:G23)</f>
         <v>0</v>
       </c>
       <c r="H22" s="26">
-        <f t="shared" si="19"/>
+        <f>SUM(H23:H23)</f>
         <v>0</v>
       </c>
       <c r="I22" s="26">
-        <f t="shared" si="19"/>
+        <f>SUM(I23:I23)</f>
         <v>0</v>
       </c>
       <c r="J22" s="26">
-        <f t="shared" si="19"/>
+        <f ca="1">SUM(J24:J24)</f>
         <v>0</v>
       </c>
       <c r="K22" s="26">
-        <f ca="1">SUM(K24:K24)</f>
+        <f>SUM(K23:K23)</f>
         <v>0</v>
       </c>
       <c r="L22" s="26">
-        <f>SUM(L23:L23)</f>
+        <f ca="1">SUM(L24:L24)</f>
         <v>0</v>
       </c>
       <c r="M22" s="26">
         <f ca="1">SUM(M24:M24)</f>
         <v>0</v>
       </c>
-      <c r="N22" s="26">
-        <f ca="1">SUM(N24:N24)</f>
-        <v>0</v>
-      </c>
-      <c r="O22" s="26"/>
-    </row>
-    <row r="23" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:15">
+      <c r="N22" s="26"/>
+    </row>
+    <row r="23" s="3" customFormat="1" ht="35.25" customHeight="1" spans="1:14">
       <c r="A23" s="21"/>
       <c r="B23" s="22"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="33"/>
-      <c r="F23" s="33"/>
-      <c r="G23" s="33"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="25"/>
+      <c r="G23" s="34"/>
       <c r="H23" s="25">
-        <f>F23+G23</f>
-        <v>0</v>
-      </c>
-      <c r="I23" s="33"/>
+        <f>F23-G23</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="25"/>
       <c r="J23" s="25">
-        <f>I23*50%</f>
-        <v>0</v>
-      </c>
-      <c r="K23" s="25">
-        <f>G23*85%</f>
-        <v>0</v>
-      </c>
-      <c r="L23" s="51">
-        <f>J23+K23</f>
-        <v>0</v>
-      </c>
-      <c r="M23" s="53"/>
-      <c r="N23" s="51">
-        <f>H23-M23</f>
-        <v>0</v>
-      </c>
-      <c r="O23" s="53"/>
-    </row>
-    <row r="24" s="6" customFormat="1" ht="33" customHeight="1" spans="1:15">
-      <c r="A24" s="34" t="s">
+        <f>H23*85%</f>
+        <v>0</v>
+      </c>
+      <c r="K23" s="27">
+        <f>I23+J23</f>
+        <v>0</v>
+      </c>
+      <c r="L23" s="28"/>
+      <c r="M23" s="27">
+        <f>F23-L23</f>
+        <v>0</v>
+      </c>
+      <c r="N23" s="28"/>
+    </row>
+    <row r="24" s="6" customFormat="1" ht="33" customHeight="1" spans="1:14">
+      <c r="A24" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="38">
+        <f>E8+E10+E12+E14+E16+E20+E22</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="38">
+        <f>F8+F10+F12+F14+F16+F20+F22</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="38">
+        <f>G8+G10+G12+G14+G16+G20+G22</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="38">
+        <f>H8+H10+H12+H14+H16+H20+H22</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="38">
+        <f t="shared" ref="I24:N24" si="17">I8+I10+I12+I14+I16+I20+I22</f>
+        <v>0</v>
+      </c>
+      <c r="J24" s="38">
+        <f ca="1" t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="K24" s="38">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="L24" s="38">
+        <f ca="1" t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="M24" s="38">
+        <f ca="1" t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="N24" s="38"/>
+    </row>
+    <row r="25" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
+      <c r="C25" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="37">
-        <f t="shared" ref="E24:O24" si="20">E8+E10+E12+E14+E16+E20+E22</f>
-        <v>0</v>
-      </c>
-      <c r="F24" s="37">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="G24" s="37">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="H24" s="37">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="I24" s="37">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="J24" s="37">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="K24" s="37">
-        <f ca="1" t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="L24" s="37">
-        <f t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="M24" s="37">
-        <f ca="1" t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="N24" s="37">
-        <f ca="1" t="shared" si="20"/>
-        <v>0</v>
-      </c>
-      <c r="O24" s="37"/>
-    </row>
-    <row r="25" s="6" customFormat="1" ht="33" customHeight="1" spans="3:18">
-      <c r="C25" s="38" t="s">
+      <c r="D25" s="39"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="40"/>
+      <c r="K25" s="57">
+        <f>K24</f>
+        <v>0</v>
+      </c>
+      <c r="L25" s="3"/>
+      <c r="M25" s="58"/>
+      <c r="N25" s="58"/>
+      <c r="O25" s="59"/>
+      <c r="Q25" s="41"/>
+    </row>
+    <row r="26" s="6" customFormat="1" ht="33" customHeight="1" spans="3:16">
+      <c r="C26" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="38"/>
-      <c r="H25" s="39"/>
-      <c r="L25" s="55">
-        <f>L24</f>
-        <v>0</v>
-      </c>
-      <c r="M25" s="3"/>
-      <c r="N25" s="56"/>
-      <c r="O25" s="56"/>
-      <c r="P25" s="57"/>
-      <c r="R25" s="59"/>
-    </row>
-    <row r="26" s="6" customFormat="1" ht="33" customHeight="1" spans="3:17">
-      <c r="C26" s="39" t="s">
+      <c r="D26" s="40"/>
+      <c r="E26" s="40"/>
+      <c r="F26" s="40"/>
+      <c r="K26" s="60">
+        <f>K25*10%</f>
+        <v>0</v>
+      </c>
+      <c r="L26" s="3"/>
+      <c r="M26" s="58"/>
+      <c r="N26" s="58"/>
+      <c r="O26" s="58"/>
+      <c r="P26" s="41"/>
+    </row>
+    <row r="27" s="6" customFormat="1" ht="33" customHeight="1" spans="3:15">
+      <c r="C27" s="40" t="s">
         <v>38</v>
       </c>
-      <c r="D26" s="39"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="39"/>
-      <c r="G26" s="39"/>
-      <c r="H26" s="39"/>
-      <c r="L26" s="58">
-        <f>L25*10%</f>
-        <v>0</v>
-      </c>
-      <c r="M26" s="3"/>
-      <c r="N26" s="56"/>
-      <c r="O26" s="56"/>
-      <c r="P26" s="56"/>
-      <c r="Q26" s="59"/>
-    </row>
-    <row r="27" s="6" customFormat="1" ht="33" customHeight="1" spans="3:16">
-      <c r="C27" s="39" t="s">
+      <c r="D27" s="40"/>
+      <c r="E27" s="40"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="41"/>
+      <c r="K27" s="60">
+        <f>K25-K26</f>
+        <v>0</v>
+      </c>
+      <c r="M27" s="58"/>
+      <c r="N27" s="58"/>
+      <c r="O27" s="58"/>
+    </row>
+    <row r="28" s="6" customFormat="1" ht="33" customHeight="1" spans="3:15">
+      <c r="C28" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="D27" s="39"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="39"/>
-      <c r="I27" s="59"/>
-      <c r="L27" s="58">
-        <f>L25-L26</f>
-        <v>0</v>
-      </c>
-      <c r="N27" s="56"/>
-      <c r="O27" s="56"/>
-      <c r="P27" s="56"/>
-    </row>
-    <row r="28" s="6" customFormat="1" ht="33" customHeight="1" spans="3:16">
-      <c r="C28" s="40" t="s">
+      <c r="D28" s="42"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="45"/>
+      <c r="I28" s="45"/>
+      <c r="J28" s="45"/>
+      <c r="K28" s="60">
+        <f ca="1">F24-K24-L24</f>
+        <v>0</v>
+      </c>
+      <c r="M28" s="58"/>
+      <c r="N28" s="58"/>
+      <c r="O28" s="58"/>
+    </row>
+    <row r="29" s="7" customFormat="1" ht="33" customHeight="1" spans="1:15">
+      <c r="A29" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="D28" s="40"/>
-      <c r="E28" s="40"/>
-      <c r="F28" s="40"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="41"/>
-      <c r="I28" s="60"/>
-      <c r="J28" s="61"/>
-      <c r="K28" s="61"/>
-      <c r="L28" s="58">
-        <f ca="1">H24-L24-M24</f>
-        <v>0</v>
-      </c>
-      <c r="N28" s="56"/>
-      <c r="O28" s="56"/>
-      <c r="P28" s="56"/>
-    </row>
-    <row r="29" s="7" customFormat="1" ht="33" customHeight="1" spans="1:16">
-      <c r="A29" s="42" t="s">
+      <c r="B29" s="46"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="46"/>
+      <c r="E29" s="47"/>
+      <c r="F29" s="48"/>
+      <c r="G29" s="48"/>
+      <c r="H29" s="48"/>
+      <c r="I29" s="48"/>
+      <c r="L29" s="41"/>
+      <c r="M29" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="B29" s="42"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="42"/>
-      <c r="E29" s="43"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="44"/>
-      <c r="I29" s="44"/>
-      <c r="J29" s="44"/>
-      <c r="M29" s="59"/>
-      <c r="N29" s="44" t="s">
-        <v>42</v>
-      </c>
-      <c r="O29" s="44"/>
-      <c r="P29" s="62"/>
+      <c r="N29" s="48"/>
+      <c r="O29" s="61"/>
     </row>
     <row r="30" s="1" customFormat="1" ht="33" customHeight="1"/>
     <row r="31" s="1" customFormat="1" ht="63" customHeight="1"/>
-    <row r="32" spans="1:15">
-      <c r="A32" s="44" t="s">
+    <row r="32" spans="1:14">
+      <c r="A32" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="B32" s="48"/>
+      <c r="C32" s="48"/>
+      <c r="D32" s="48"/>
+      <c r="M32" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="B32" s="44"/>
-      <c r="C32" s="44"/>
-      <c r="D32" s="44"/>
-      <c r="N32" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="O32" s="44"/>
-    </row>
-    <row r="33" s="1" customFormat="1" spans="18:18">
-      <c r="R33" s="64"/>
-    </row>
-    <row r="36" s="1" customFormat="1" spans="7:11">
-      <c r="G36" s="44"/>
-      <c r="H36" s="44"/>
-      <c r="I36" s="44"/>
-      <c r="J36" s="44"/>
-      <c r="K36" s="7"/>
-    </row>
-    <row r="37" s="3" customFormat="1" spans="3:14">
-      <c r="C37" s="45"/>
-      <c r="D37" s="45"/>
-      <c r="E37" s="45"/>
-      <c r="F37" s="45"/>
-      <c r="G37" s="45"/>
-      <c r="H37" s="45"/>
-      <c r="N37" s="63"/>
+      <c r="N32" s="48"/>
+    </row>
+    <row r="33" s="1" customFormat="1" spans="17:17">
+      <c r="Q33" s="63"/>
+    </row>
+    <row r="36" s="1" customFormat="1" spans="6:10">
+      <c r="F36" s="48"/>
+      <c r="G36" s="48"/>
+      <c r="H36" s="48"/>
+      <c r="I36" s="48"/>
+      <c r="J36" s="7"/>
+    </row>
+    <row r="37" s="3" customFormat="1" spans="3:13">
+      <c r="C37" s="49"/>
+      <c r="D37" s="49"/>
+      <c r="E37" s="49"/>
+      <c r="F37" s="49"/>
+      <c r="M37" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="D1:E1"/>
     <mergeCell ref="A24:D24"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="C26:G26"/>
-    <mergeCell ref="C27:G27"/>
-    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="C28:E28"/>
     <mergeCell ref="A29:D29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="M29:N29"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="G36:J36"/>
-    <mergeCell ref="C37:G37"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="F36:I36"/>
+    <mergeCell ref="C37:E37"/>
   </mergeCells>
   <conditionalFormatting sqref="C7">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>

</xml_diff>